<commit_message>
Atualiza lista de CADIFAs deferidas (execução automática 10/08/2026)
2 novas CADIFAs desde a última execução: empagliflozina (Metrochem Api
Private Limited) e semaglutida (Sinopep-Allsino Biopharmaceutical Co.).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014q1XhEFwoBNrFsv6ikdSjJ
</commit_message>
<xml_diff>
--- a/cadifa_completo.xlsx
+++ b/cadifa_completo.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E582"/>
+  <dimension ref="A1:E581"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1784,7 +1784,7 @@
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>001</t>
+          <t>001.1</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
@@ -2567,7 +2567,7 @@
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>001</t>
+          <t>001.1</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
@@ -3524,7 +3524,7 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>Synthimed Labs Private Limited</t>
+          <t>Ind-Swift Laboratories Limited</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
@@ -5090,7 +5090,7 @@
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>Synthimed Labs Private Limited</t>
+          <t>Ind-Swift Laboratories Limited</t>
         </is>
       </c>
       <c r="B174" t="inlineStr">
@@ -11354,7 +11354,7 @@
     <row r="406">
       <c r="A406" t="inlineStr">
         <is>
-          <t>Anlon Health Care Pvt Ltd</t>
+          <t>Anlon Healthcare Limited</t>
         </is>
       </c>
       <c r="B406" t="inlineStr">
@@ -13892,71 +13892,71 @@
     <row r="500">
       <c r="A500" t="inlineStr">
         <is>
-          <t>Synthon Bv</t>
+          <t>Fdc Limited</t>
         </is>
       </c>
       <c r="B500" t="inlineStr">
         <is>
-          <t>sugamadex sódico</t>
+          <t>maleato de timolol</t>
         </is>
       </c>
       <c r="C500" t="inlineStr">
         <is>
-          <t>25351779849202193</t>
+          <t>25351087503202246</t>
         </is>
       </c>
       <c r="D500" t="inlineStr">
         <is>
-          <t>002</t>
+          <t>001</t>
         </is>
       </c>
       <c r="E500" t="inlineStr">
         <is>
-          <t>13/11/2023</t>
+          <t>09/11/2023</t>
         </is>
       </c>
     </row>
     <row r="501">
       <c r="A501" t="inlineStr">
         <is>
-          <t>Fdc Limited</t>
+          <t>Medichem S.A.</t>
         </is>
       </c>
       <c r="B501" t="inlineStr">
         <is>
-          <t>maleato de timolol</t>
+          <t>micafungina sódica</t>
         </is>
       </c>
       <c r="C501" t="inlineStr">
         <is>
-          <t>25351087503202246</t>
+          <t>25351543525202208</t>
         </is>
       </c>
       <c r="D501" t="inlineStr">
         <is>
-          <t>001</t>
+          <t>002</t>
         </is>
       </c>
       <c r="E501" t="inlineStr">
         <is>
-          <t>09/11/2023</t>
+          <t>06/11/2023</t>
         </is>
       </c>
     </row>
     <row r="502">
       <c r="A502" t="inlineStr">
         <is>
-          <t>Medichem S.A.</t>
+          <t>Harman Finochem Limited</t>
         </is>
       </c>
       <c r="B502" t="inlineStr">
         <is>
-          <t>micafungina sódica</t>
+          <t>fenitoína</t>
         </is>
       </c>
       <c r="C502" t="inlineStr">
         <is>
-          <t>25351543525202208</t>
+          <t>25351122886202214</t>
         </is>
       </c>
       <c r="D502" t="inlineStr">
@@ -13966,24 +13966,24 @@
       </c>
       <c r="E502" t="inlineStr">
         <is>
-          <t>06/11/2023</t>
+          <t>03/11/2023</t>
         </is>
       </c>
     </row>
     <row r="503">
       <c r="A503" t="inlineStr">
         <is>
-          <t>Harman Finochem Limited</t>
+          <t>Nortec Química S.A</t>
         </is>
       </c>
       <c r="B503" t="inlineStr">
         <is>
-          <t>fenitoína</t>
+          <t>micofenolato de sódio</t>
         </is>
       </c>
       <c r="C503" t="inlineStr">
         <is>
-          <t>25351122886202214</t>
+          <t>25351448083202289</t>
         </is>
       </c>
       <c r="D503" t="inlineStr">
@@ -14000,49 +14000,49 @@
     <row r="504">
       <c r="A504" t="inlineStr">
         <is>
-          <t>Nortec Química S.A</t>
+          <t>Emcure Pharmaceuticals Limited</t>
         </is>
       </c>
       <c r="B504" t="inlineStr">
         <is>
-          <t>micofenolato de sódio</t>
+          <t>milrinona</t>
         </is>
       </c>
       <c r="C504" t="inlineStr">
         <is>
-          <t>25351448083202289</t>
+          <t>25351038756202296</t>
         </is>
       </c>
       <c r="D504" t="inlineStr">
         <is>
-          <t>002</t>
+          <t>001</t>
         </is>
       </c>
       <c r="E504" t="inlineStr">
         <is>
-          <t>03/11/2023</t>
+          <t>30/10/2023</t>
         </is>
       </c>
     </row>
     <row r="505">
       <c r="A505" t="inlineStr">
         <is>
-          <t>Emcure Pharmaceuticals Limited</t>
+          <t>Neuland Laboratories Limited</t>
         </is>
       </c>
       <c r="B505" t="inlineStr">
         <is>
-          <t>milrinona</t>
+          <t>mirtazapina</t>
         </is>
       </c>
       <c r="C505" t="inlineStr">
         <is>
-          <t>25351038756202296</t>
+          <t>25351589465202261</t>
         </is>
       </c>
       <c r="D505" t="inlineStr">
         <is>
-          <t>001</t>
+          <t>003</t>
         </is>
       </c>
       <c r="E505" t="inlineStr">
@@ -14054,44 +14054,44 @@
     <row r="506">
       <c r="A506" t="inlineStr">
         <is>
-          <t>Neuland Laboratories Limited</t>
+          <t>Ctx Lifesciences Pvt. Ltd.</t>
         </is>
       </c>
       <c r="B506" t="inlineStr">
         <is>
-          <t>mirtazapina</t>
+          <t>succinato de metoprolol</t>
         </is>
       </c>
       <c r="C506" t="inlineStr">
         <is>
-          <t>25351589465202261</t>
+          <t>25351287504202116</t>
         </is>
       </c>
       <c r="D506" t="inlineStr">
         <is>
-          <t>003</t>
+          <t>001</t>
         </is>
       </c>
       <c r="E506" t="inlineStr">
         <is>
-          <t>30/10/2023</t>
+          <t>27/10/2023</t>
         </is>
       </c>
     </row>
     <row r="507">
       <c r="A507" t="inlineStr">
         <is>
-          <t>Ctx Lifesciences Pvt. Ltd.</t>
+          <t>Ulkar Kimya Sanayii Ve Ticaret A.S.</t>
         </is>
       </c>
       <c r="B507" t="inlineStr">
         <is>
-          <t>succinato de metoprolol</t>
+          <t>etodolaco</t>
         </is>
       </c>
       <c r="C507" t="inlineStr">
         <is>
-          <t>25351287504202116</t>
+          <t>25351171112202217</t>
         </is>
       </c>
       <c r="D507" t="inlineStr">
@@ -14101,29 +14101,29 @@
       </c>
       <c r="E507" t="inlineStr">
         <is>
-          <t>27/10/2023</t>
+          <t>25/10/2023</t>
         </is>
       </c>
     </row>
     <row r="508">
       <c r="A508" t="inlineStr">
         <is>
-          <t>Ulkar Kimya Sanayii Ve Ticaret A.S.</t>
+          <t>Msn Pharmachem Private Limited</t>
         </is>
       </c>
       <c r="B508" t="inlineStr">
         <is>
-          <t>etodolaco</t>
+          <t>vildagliptina</t>
         </is>
       </c>
       <c r="C508" t="inlineStr">
         <is>
-          <t>25351171112202217</t>
+          <t>25351407050202289</t>
         </is>
       </c>
       <c r="D508" t="inlineStr">
         <is>
-          <t>001</t>
+          <t>002</t>
         </is>
       </c>
       <c r="E508" t="inlineStr">
@@ -14135,22 +14135,22 @@
     <row r="509">
       <c r="A509" t="inlineStr">
         <is>
-          <t>Msn Pharmachem Private Limited</t>
+          <t>Cohance Lifesciences Limited</t>
         </is>
       </c>
       <c r="B509" t="inlineStr">
         <is>
-          <t>vildagliptina</t>
+          <t>lamotrigina</t>
         </is>
       </c>
       <c r="C509" t="inlineStr">
         <is>
-          <t>25351407050202289</t>
+          <t>25351699210202125</t>
         </is>
       </c>
       <c r="D509" t="inlineStr">
         <is>
-          <t>002</t>
+          <t>001</t>
         </is>
       </c>
       <c r="E509" t="inlineStr">
@@ -14162,17 +14162,17 @@
     <row r="510">
       <c r="A510" t="inlineStr">
         <is>
-          <t>Cohance Lifesciences Limited</t>
+          <t>Hubei Yitai Pharmaceutical Co., Ltd.</t>
         </is>
       </c>
       <c r="B510" t="inlineStr">
         <is>
-          <t>lamotrigina</t>
+          <t>aciclovir</t>
         </is>
       </c>
       <c r="C510" t="inlineStr">
         <is>
-          <t>25351699210202125</t>
+          <t>25351473051202131</t>
         </is>
       </c>
       <c r="D510" t="inlineStr">
@@ -14182,29 +14182,29 @@
       </c>
       <c r="E510" t="inlineStr">
         <is>
-          <t>25/10/2023</t>
+          <t>24/10/2023</t>
         </is>
       </c>
     </row>
     <row r="511">
       <c r="A511" t="inlineStr">
         <is>
-          <t>Hubei Yitai Pharmaceutical Co., Ltd.</t>
+          <t>Janssen-Cilag Farmaceutica Ltda</t>
         </is>
       </c>
       <c r="B511" t="inlineStr">
         <is>
-          <t>aciclovir</t>
+          <t>etanolato de darunavir</t>
         </is>
       </c>
       <c r="C511" t="inlineStr">
         <is>
-          <t>25351473051202131</t>
+          <t>25351122285202201</t>
         </is>
       </c>
       <c r="D511" t="inlineStr">
         <is>
-          <t>001</t>
+          <t>002</t>
         </is>
       </c>
       <c r="E511" t="inlineStr">
@@ -14216,17 +14216,17 @@
     <row r="512">
       <c r="A512" t="inlineStr">
         <is>
-          <t>Janssen-Cilag Farmaceutica Ltda</t>
+          <t>Torrent Pharmaceuticals Limited</t>
         </is>
       </c>
       <c r="B512" t="inlineStr">
         <is>
-          <t>etanolato de darunavir</t>
+          <t>lamotrigina</t>
         </is>
       </c>
       <c r="C512" t="inlineStr">
         <is>
-          <t>25351122285202201</t>
+          <t>25351171478202288</t>
         </is>
       </c>
       <c r="D512" t="inlineStr">
@@ -14236,56 +14236,56 @@
       </c>
       <c r="E512" t="inlineStr">
         <is>
-          <t>24/10/2023</t>
+          <t>23/10/2023</t>
         </is>
       </c>
     </row>
     <row r="513">
       <c r="A513" t="inlineStr">
         <is>
-          <t>Torrent Pharmaceuticals Limited</t>
+          <t>Wuhan Wuyao Pharmaceutical Co., Ltd.</t>
         </is>
       </c>
       <c r="B513" t="inlineStr">
         <is>
-          <t>lamotrigina</t>
+          <t>dipirona monoidratada</t>
         </is>
       </c>
       <c r="C513" t="inlineStr">
         <is>
-          <t>25351171478202288</t>
+          <t>25351596512202223</t>
         </is>
       </c>
       <c r="D513" t="inlineStr">
         <is>
-          <t>002</t>
+          <t>001</t>
         </is>
       </c>
       <c r="E513" t="inlineStr">
         <is>
-          <t>23/10/2023</t>
+          <t>11/10/2023</t>
         </is>
       </c>
     </row>
     <row r="514">
       <c r="A514" t="inlineStr">
         <is>
-          <t>Wuhan Wuyao Pharmaceutical Co., Ltd.</t>
+          <t>Tapi Brazil Ltda</t>
         </is>
       </c>
       <c r="B514" t="inlineStr">
         <is>
-          <t>dipirona monoidratada</t>
+          <t>dasatinibe monoidratado</t>
         </is>
       </c>
       <c r="C514" t="inlineStr">
         <is>
-          <t>25351596512202223</t>
+          <t>25351543510202231</t>
         </is>
       </c>
       <c r="D514" t="inlineStr">
         <is>
-          <t>001</t>
+          <t>002.1</t>
         </is>
       </c>
       <c r="E514" t="inlineStr">
@@ -14297,44 +14297,44 @@
     <row r="515">
       <c r="A515" t="inlineStr">
         <is>
-          <t>Tapi Brazil Ltda</t>
+          <t>Sun Pharmaceutical Industries Limited</t>
         </is>
       </c>
       <c r="B515" t="inlineStr">
         <is>
-          <t>dasatinibe monoidratado</t>
+          <t>cloridrato de donepezila monoidratado</t>
         </is>
       </c>
       <c r="C515" t="inlineStr">
         <is>
-          <t>25351543510202231</t>
+          <t>25351244345202238</t>
         </is>
       </c>
       <c r="D515" t="inlineStr">
         <is>
-          <t>002.1</t>
+          <t>001</t>
         </is>
       </c>
       <c r="E515" t="inlineStr">
         <is>
-          <t>11/10/2023</t>
+          <t>05/10/2023</t>
         </is>
       </c>
     </row>
     <row r="516">
       <c r="A516" t="inlineStr">
         <is>
-          <t>Sun Pharmaceutical Industries Limited</t>
+          <t>Zhejiang Hisun Pharmaceutical Co., Ltd.</t>
         </is>
       </c>
       <c r="B516" t="inlineStr">
         <is>
-          <t>cloridrato de donepezila monoidratado</t>
+          <t>adenosina</t>
         </is>
       </c>
       <c r="C516" t="inlineStr">
         <is>
-          <t>25351244345202238</t>
+          <t>25351008874202199</t>
         </is>
       </c>
       <c r="D516" t="inlineStr">
@@ -14344,29 +14344,29 @@
       </c>
       <c r="E516" t="inlineStr">
         <is>
-          <t>05/10/2023</t>
+          <t>03/10/2023</t>
         </is>
       </c>
     </row>
     <row r="517">
       <c r="A517" t="inlineStr">
         <is>
-          <t>Zhejiang Hisun Pharmaceutical Co., Ltd.</t>
+          <t>Moehs Ibérica, S.L.</t>
         </is>
       </c>
       <c r="B517" t="inlineStr">
         <is>
-          <t>adenosina</t>
+          <t>hemifumarato de bisoprolol</t>
         </is>
       </c>
       <c r="C517" t="inlineStr">
         <is>
-          <t>25351008874202199</t>
+          <t>25351618932202197</t>
         </is>
       </c>
       <c r="D517" t="inlineStr">
         <is>
-          <t>001</t>
+          <t>002.1</t>
         </is>
       </c>
       <c r="E517" t="inlineStr">
@@ -14378,49 +14378,49 @@
     <row r="518">
       <c r="A518" t="inlineStr">
         <is>
-          <t>Moehs Ibérica, S.L.</t>
+          <t>Tapi Brazil Ltda</t>
         </is>
       </c>
       <c r="B518" t="inlineStr">
         <is>
-          <t>hemifumarato de bisoprolol</t>
+          <t>rivaroxabana</t>
         </is>
       </c>
       <c r="C518" t="inlineStr">
         <is>
-          <t>25351618932202197</t>
+          <t>25351312133202291</t>
         </is>
       </c>
       <c r="D518" t="inlineStr">
         <is>
-          <t>002.1</t>
+          <t>003</t>
         </is>
       </c>
       <c r="E518" t="inlineStr">
         <is>
-          <t>03/10/2023</t>
+          <t>26/09/2023</t>
         </is>
       </c>
     </row>
     <row r="519">
       <c r="A519" t="inlineStr">
         <is>
-          <t>Tapi Brazil Ltda</t>
+          <t>Shilpa Pharma Lifesciences Limited</t>
         </is>
       </c>
       <c r="B519" t="inlineStr">
         <is>
-          <t>rivaroxabana</t>
+          <t>bortezomibe</t>
         </is>
       </c>
       <c r="C519" t="inlineStr">
         <is>
-          <t>25351312133202291</t>
+          <t>25351839141202107</t>
         </is>
       </c>
       <c r="D519" t="inlineStr">
         <is>
-          <t>003</t>
+          <t>001</t>
         </is>
       </c>
       <c r="E519" t="inlineStr">
@@ -14432,22 +14432,22 @@
     <row r="520">
       <c r="A520" t="inlineStr">
         <is>
-          <t>Shilpa Pharma Lifesciences Limited</t>
+          <t>Dr Reddys Farmacêutica Do Brasil Ltda</t>
         </is>
       </c>
       <c r="B520" t="inlineStr">
         <is>
-          <t>bortezomibe</t>
+          <t>lenalidomida</t>
         </is>
       </c>
       <c r="C520" t="inlineStr">
         <is>
-          <t>25351839141202107</t>
+          <t>25351068660202252</t>
         </is>
       </c>
       <c r="D520" t="inlineStr">
         <is>
-          <t>001</t>
+          <t>003</t>
         </is>
       </c>
       <c r="E520" t="inlineStr">
@@ -14459,49 +14459,49 @@
     <row r="521">
       <c r="A521" t="inlineStr">
         <is>
-          <t>Dr Reddys Farmacêutica Do Brasil Ltda</t>
+          <t>Zhuhai United Laboratories Co., Ltd.</t>
         </is>
       </c>
       <c r="B521" t="inlineStr">
         <is>
-          <t>lenalidomida</t>
+          <t>ampicilina sódica</t>
         </is>
       </c>
       <c r="C521" t="inlineStr">
         <is>
-          <t>25351068660202252</t>
+          <t>25351433410202117</t>
         </is>
       </c>
       <c r="D521" t="inlineStr">
         <is>
-          <t>003</t>
+          <t>002.1</t>
         </is>
       </c>
       <c r="E521" t="inlineStr">
         <is>
-          <t>26/09/2023</t>
+          <t>22/09/2023</t>
         </is>
       </c>
     </row>
     <row r="522">
       <c r="A522" t="inlineStr">
         <is>
-          <t>Zhuhai United Laboratories Co., Ltd.</t>
+          <t>Chemwerth, Inc.</t>
         </is>
       </c>
       <c r="B522" t="inlineStr">
         <is>
-          <t>ampicilina sódica</t>
+          <t>milrinona</t>
         </is>
       </c>
       <c r="C522" t="inlineStr">
         <is>
-          <t>25351433410202117</t>
+          <t>25351869642202118</t>
         </is>
       </c>
       <c r="D522" t="inlineStr">
         <is>
-          <t>002.1</t>
+          <t>001.1</t>
         </is>
       </c>
       <c r="E522" t="inlineStr">
@@ -14513,17 +14513,17 @@
     <row r="523">
       <c r="A523" t="inlineStr">
         <is>
-          <t>Chemwerth, Inc.</t>
+          <t>Msn Pharmachem Private Limited</t>
         </is>
       </c>
       <c r="B523" t="inlineStr">
         <is>
-          <t>milrinona</t>
+          <t>bromidrato de vortioxetina</t>
         </is>
       </c>
       <c r="C523" t="inlineStr">
         <is>
-          <t>25351869642202118</t>
+          <t>25351252213202280</t>
         </is>
       </c>
       <c r="D523" t="inlineStr">
@@ -14533,83 +14533,83 @@
       </c>
       <c r="E523" t="inlineStr">
         <is>
-          <t>22/09/2023</t>
+          <t>18/09/2023</t>
         </is>
       </c>
     </row>
     <row r="524">
       <c r="A524" t="inlineStr">
         <is>
-          <t>Msn Pharmachem Private Limited</t>
+          <t>Matrix Pharmacorp Private Limited</t>
         </is>
       </c>
       <c r="B524" t="inlineStr">
         <is>
-          <t>bromidrato de vortioxetina</t>
+          <t>hemitartarato de zolpidem</t>
         </is>
       </c>
       <c r="C524" t="inlineStr">
         <is>
-          <t>25351252213202280</t>
+          <t>25351580744202189</t>
         </is>
       </c>
       <c r="D524" t="inlineStr">
         <is>
-          <t>001.1</t>
+          <t>003</t>
         </is>
       </c>
       <c r="E524" t="inlineStr">
         <is>
-          <t>18/09/2023</t>
+          <t>08/09/2023</t>
         </is>
       </c>
     </row>
     <row r="525">
       <c r="A525" t="inlineStr">
         <is>
-          <t>Matrix Pharmacorp Private Limited</t>
+          <t>Msn Pharmachem Private Limited</t>
         </is>
       </c>
       <c r="B525" t="inlineStr">
         <is>
-          <t>hemitartarato de zolpidem</t>
+          <t>aripiprazol</t>
         </is>
       </c>
       <c r="C525" t="inlineStr">
         <is>
-          <t>25351580744202189</t>
+          <t>25351524957202210</t>
         </is>
       </c>
       <c r="D525" t="inlineStr">
         <is>
-          <t>003</t>
+          <t>002</t>
         </is>
       </c>
       <c r="E525" t="inlineStr">
         <is>
-          <t>08/09/2023</t>
+          <t>05/09/2023</t>
         </is>
       </c>
     </row>
     <row r="526">
       <c r="A526" t="inlineStr">
         <is>
-          <t>Msn Pharmachem Private Limited</t>
+          <t>Sun Pharmaceutical Industries Limited</t>
         </is>
       </c>
       <c r="B526" t="inlineStr">
         <is>
-          <t>aripiprazol</t>
+          <t>mesilato de lenvatinibe</t>
         </is>
       </c>
       <c r="C526" t="inlineStr">
         <is>
-          <t>25351524957202210</t>
+          <t>25351206913202201</t>
         </is>
       </c>
       <c r="D526" t="inlineStr">
         <is>
-          <t>002</t>
+          <t>001</t>
         </is>
       </c>
       <c r="E526" t="inlineStr">
@@ -14621,17 +14621,17 @@
     <row r="527">
       <c r="A527" t="inlineStr">
         <is>
-          <t>Sun Pharmaceutical Industries Limited</t>
+          <t>Dr Reddys Farmacêutica Do Brasil Ltda</t>
         </is>
       </c>
       <c r="B527" t="inlineStr">
         <is>
-          <t>mesilato de lenvatinibe</t>
+          <t>cloridrato de naratriptana</t>
         </is>
       </c>
       <c r="C527" t="inlineStr">
         <is>
-          <t>25351206913202201</t>
+          <t>25351673613202225</t>
         </is>
       </c>
       <c r="D527" t="inlineStr">
@@ -14648,17 +14648,17 @@
     <row r="528">
       <c r="A528" t="inlineStr">
         <is>
-          <t>Dr Reddys Farmacêutica Do Brasil Ltda</t>
+          <t>Intas Pharmaceuticals Limited</t>
         </is>
       </c>
       <c r="B528" t="inlineStr">
         <is>
-          <t>cloridrato de naratriptana</t>
+          <t>carfilzomibe</t>
         </is>
       </c>
       <c r="C528" t="inlineStr">
         <is>
-          <t>25351673613202225</t>
+          <t>25351255810202185</t>
         </is>
       </c>
       <c r="D528" t="inlineStr">
@@ -14668,78 +14668,78 @@
       </c>
       <c r="E528" t="inlineStr">
         <is>
-          <t>05/09/2023</t>
+          <t>31/08/2023</t>
         </is>
       </c>
     </row>
     <row r="529">
       <c r="A529" t="inlineStr">
         <is>
-          <t>Intas Pharmaceuticals Limited</t>
+          <t>Scl Lifesciences Limited</t>
         </is>
       </c>
       <c r="B529" t="inlineStr">
         <is>
-          <t>carfilzomibe</t>
+          <t>trometamol cetorolaco</t>
         </is>
       </c>
       <c r="C529" t="inlineStr">
         <is>
-          <t>25351255810202185</t>
+          <t>25351654225202164</t>
         </is>
       </c>
       <c r="D529" t="inlineStr">
         <is>
-          <t>001</t>
+          <t>002</t>
         </is>
       </c>
       <c r="E529" t="inlineStr">
         <is>
-          <t>31/08/2023</t>
+          <t>29/08/2023</t>
         </is>
       </c>
     </row>
     <row r="530">
       <c r="A530" t="inlineStr">
         <is>
-          <t>Scl Lifesciences Limited</t>
+          <t>Msn Laboratories Private Limited</t>
         </is>
       </c>
       <c r="B530" t="inlineStr">
         <is>
-          <t>trometamol cetorolaco</t>
+          <t>pitavastatina cálcica pentaidratada</t>
         </is>
       </c>
       <c r="C530" t="inlineStr">
         <is>
-          <t>25351654225202164</t>
+          <t>25351527145202218</t>
         </is>
       </c>
       <c r="D530" t="inlineStr">
         <is>
-          <t>002</t>
+          <t>001</t>
         </is>
       </c>
       <c r="E530" t="inlineStr">
         <is>
-          <t>29/08/2023</t>
+          <t>28/08/2023</t>
         </is>
       </c>
     </row>
     <row r="531">
       <c r="A531" t="inlineStr">
         <is>
-          <t>Msn Laboratories Private Limited</t>
+          <t>Glochem Industries Private Limited</t>
         </is>
       </c>
       <c r="B531" t="inlineStr">
         <is>
-          <t>pitavastatina cálcica pentaidratada</t>
+          <t>besilato de levanlodipino hemipentaidratado</t>
         </is>
       </c>
       <c r="C531" t="inlineStr">
         <is>
-          <t>25351527145202218</t>
+          <t>25351492777202253</t>
         </is>
       </c>
       <c r="D531" t="inlineStr">
@@ -14749,24 +14749,24 @@
       </c>
       <c r="E531" t="inlineStr">
         <is>
-          <t>28/08/2023</t>
+          <t>23/08/2023</t>
         </is>
       </c>
     </row>
     <row r="532">
       <c r="A532" t="inlineStr">
         <is>
-          <t>Glochem Industries Private Limited</t>
+          <t>Ipca Laboratories Ltd.</t>
         </is>
       </c>
       <c r="B532" t="inlineStr">
         <is>
-          <t>besilato de levanlodipino hemipentaidratado</t>
+          <t>hidroclorotiazida</t>
         </is>
       </c>
       <c r="C532" t="inlineStr">
         <is>
-          <t>25351492777202253</t>
+          <t>25351234613202211</t>
         </is>
       </c>
       <c r="D532" t="inlineStr">
@@ -14776,24 +14776,24 @@
       </c>
       <c r="E532" t="inlineStr">
         <is>
-          <t>23/08/2023</t>
+          <t>22/08/2023</t>
         </is>
       </c>
     </row>
     <row r="533">
       <c r="A533" t="inlineStr">
         <is>
-          <t>Ipca Laboratories Ltd.</t>
+          <t>Centrient Pharmaceuticals Spain, S.A.</t>
         </is>
       </c>
       <c r="B533" t="inlineStr">
         <is>
-          <t>hidroclorotiazida</t>
+          <t>cefalexina monoidratada</t>
         </is>
       </c>
       <c r="C533" t="inlineStr">
         <is>
-          <t>25351234613202211</t>
+          <t>25351196266202122</t>
         </is>
       </c>
       <c r="D533" t="inlineStr">
@@ -14803,88 +14803,88 @@
       </c>
       <c r="E533" t="inlineStr">
         <is>
-          <t>22/08/2023</t>
+          <t>17/08/2023</t>
         </is>
       </c>
     </row>
     <row r="534">
       <c r="A534" t="inlineStr">
         <is>
-          <t>Centrient Pharmaceuticals Spain, S.A.</t>
+          <t>Matrix Pharmacorp Private Limited</t>
         </is>
       </c>
       <c r="B534" t="inlineStr">
         <is>
-          <t>cefalexina monoidratada</t>
+          <t>aciclovir</t>
         </is>
       </c>
       <c r="C534" t="inlineStr">
         <is>
-          <t>25351196266202122</t>
+          <t>25351247888202126</t>
         </is>
       </c>
       <c r="D534" t="inlineStr">
         <is>
-          <t>001</t>
+          <t>004</t>
         </is>
       </c>
       <c r="E534" t="inlineStr">
         <is>
-          <t>17/08/2023</t>
+          <t>04/08/2023</t>
         </is>
       </c>
     </row>
     <row r="535">
       <c r="A535" t="inlineStr">
         <is>
-          <t>Matrix Pharmacorp Private Limited</t>
+          <t>Solara Active Pharma Sciences Limited</t>
         </is>
       </c>
       <c r="B535" t="inlineStr">
         <is>
-          <t>aciclovir</t>
+          <t>ibuprofeno</t>
         </is>
       </c>
       <c r="C535" t="inlineStr">
         <is>
-          <t>25351247888202126</t>
+          <t>25351072240202351</t>
         </is>
       </c>
       <c r="D535" t="inlineStr">
         <is>
-          <t>004</t>
+          <t>001.1</t>
         </is>
       </c>
       <c r="E535" t="inlineStr">
         <is>
-          <t>04/08/2023</t>
+          <t>14/07/2023</t>
         </is>
       </c>
     </row>
     <row r="536">
       <c r="A536" t="inlineStr">
         <is>
-          <t>Solara Active Pharma Sciences Limited</t>
+          <t>Harman Finochem Limited</t>
         </is>
       </c>
       <c r="B536" t="inlineStr">
         <is>
-          <t>ibuprofeno</t>
+          <t>cloridrato de metformina</t>
         </is>
       </c>
       <c r="C536" t="inlineStr">
         <is>
-          <t>25351072240202351</t>
+          <t>25351583229202231</t>
         </is>
       </c>
       <c r="D536" t="inlineStr">
         <is>
-          <t>001.1</t>
+          <t>001</t>
         </is>
       </c>
       <c r="E536" t="inlineStr">
         <is>
-          <t>14/07/2023</t>
+          <t>11/07/2023</t>
         </is>
       </c>
     </row>
@@ -14901,7 +14901,7 @@
       </c>
       <c r="C537" t="inlineStr">
         <is>
-          <t>25351583229202231</t>
+          <t>25351165919202211</t>
         </is>
       </c>
       <c r="D537" t="inlineStr">
@@ -14911,29 +14911,29 @@
       </c>
       <c r="E537" t="inlineStr">
         <is>
-          <t>11/07/2023</t>
+          <t>06/07/2023</t>
         </is>
       </c>
     </row>
     <row r="538">
       <c r="A538" t="inlineStr">
         <is>
-          <t>Harman Finochem Limited</t>
+          <t>Msn Organics Private Limited</t>
         </is>
       </c>
       <c r="B538" t="inlineStr">
         <is>
-          <t>cloridrato de metformina</t>
+          <t>parecoxibe sódico</t>
         </is>
       </c>
       <c r="C538" t="inlineStr">
         <is>
-          <t>25351165919202211</t>
+          <t>25351000511202296</t>
         </is>
       </c>
       <c r="D538" t="inlineStr">
         <is>
-          <t>001</t>
+          <t>002</t>
         </is>
       </c>
       <c r="E538" t="inlineStr">
@@ -14945,17 +14945,17 @@
     <row r="539">
       <c r="A539" t="inlineStr">
         <is>
-          <t>Msn Organics Private Limited</t>
+          <t>Msn Pharmachem Private Limited</t>
         </is>
       </c>
       <c r="B539" t="inlineStr">
         <is>
-          <t>parecoxibe sódico</t>
+          <t>fosfato de sitagliptina monoidratado</t>
         </is>
       </c>
       <c r="C539" t="inlineStr">
         <is>
-          <t>25351000511202296</t>
+          <t>25351745532202153</t>
         </is>
       </c>
       <c r="D539" t="inlineStr">
@@ -14965,267 +14965,267 @@
       </c>
       <c r="E539" t="inlineStr">
         <is>
-          <t>06/07/2023</t>
+          <t>23/06/2023</t>
         </is>
       </c>
     </row>
     <row r="540">
       <c r="A540" t="inlineStr">
         <is>
-          <t>Msn Pharmachem Private Limited</t>
+          <t>Alivus Life Sciences Limited</t>
         </is>
       </c>
       <c r="B540" t="inlineStr">
         <is>
-          <t>fosfato de sitagliptina monoidratado</t>
+          <t>hemitartarato de zolpidem</t>
         </is>
       </c>
       <c r="C540" t="inlineStr">
         <is>
-          <t>25351745532202153</t>
+          <t>25351851362202145</t>
         </is>
       </c>
       <c r="D540" t="inlineStr">
         <is>
-          <t>002</t>
+          <t>003</t>
         </is>
       </c>
       <c r="E540" t="inlineStr">
         <is>
-          <t>23/06/2023</t>
+          <t>20/06/2023</t>
         </is>
       </c>
     </row>
     <row r="541">
       <c r="A541" t="inlineStr">
         <is>
-          <t>Alivus Life Sciences Limited</t>
+          <t>Macfarlan Smith Limited</t>
         </is>
       </c>
       <c r="B541" t="inlineStr">
         <is>
-          <t>hemitartarato de zolpidem</t>
+          <t>fosfato de codeína hemi-hidratado</t>
         </is>
       </c>
       <c r="C541" t="inlineStr">
         <is>
-          <t>25351851362202145</t>
+          <t>25351214747202127</t>
         </is>
       </c>
       <c r="D541" t="inlineStr">
         <is>
-          <t>003</t>
+          <t>001</t>
         </is>
       </c>
       <c r="E541" t="inlineStr">
         <is>
-          <t>20/06/2023</t>
+          <t>30/05/2023</t>
         </is>
       </c>
     </row>
     <row r="542">
       <c r="A542" t="inlineStr">
         <is>
-          <t>Macfarlan Smith Limited</t>
+          <t>Aspen Oss B.V.</t>
         </is>
       </c>
       <c r="B542" t="inlineStr">
         <is>
-          <t>fosfato de codeína hemi-hidratado</t>
+          <t>ocitocina</t>
         </is>
       </c>
       <c r="C542" t="inlineStr">
         <is>
-          <t>25351214747202127</t>
+          <t>25351762016202193</t>
         </is>
       </c>
       <c r="D542" t="inlineStr">
         <is>
-          <t>001</t>
+          <t>002</t>
         </is>
       </c>
       <c r="E542" t="inlineStr">
         <is>
-          <t>30/05/2023</t>
+          <t>29/05/2023</t>
         </is>
       </c>
     </row>
     <row r="543">
       <c r="A543" t="inlineStr">
         <is>
-          <t>Aspen Oss B.V.</t>
+          <t>Sinopharm Weiqida Pharmaceutical Co., Ltd.</t>
         </is>
       </c>
       <c r="B543" t="inlineStr">
         <is>
-          <t>ocitocina</t>
+          <t>ceftriaxona dissódica hemieptaidratada</t>
         </is>
       </c>
       <c r="C543" t="inlineStr">
         <is>
-          <t>25351762016202193</t>
+          <t>25351464371202108</t>
         </is>
       </c>
       <c r="D543" t="inlineStr">
         <is>
-          <t>002</t>
+          <t>001</t>
         </is>
       </c>
       <c r="E543" t="inlineStr">
         <is>
-          <t>29/05/2023</t>
+          <t>26/05/2023</t>
         </is>
       </c>
     </row>
     <row r="544">
       <c r="A544" t="inlineStr">
         <is>
-          <t>Sinopharm Weiqida Pharmaceutical Co., Ltd.</t>
+          <t>Chemo Do Brasil Comércio De Farmoquímicos Ltda</t>
         </is>
       </c>
       <c r="B544" t="inlineStr">
         <is>
-          <t>ceftriaxona dissódica hemieptaidratada</t>
+          <t>drospirenona</t>
         </is>
       </c>
       <c r="C544" t="inlineStr">
         <is>
-          <t>25351464371202108</t>
+          <t>25351273206202211</t>
         </is>
       </c>
       <c r="D544" t="inlineStr">
         <is>
-          <t>001</t>
+          <t>005</t>
         </is>
       </c>
       <c r="E544" t="inlineStr">
         <is>
-          <t>26/05/2023</t>
+          <t>23/05/2023</t>
         </is>
       </c>
     </row>
     <row r="545">
       <c r="A545" t="inlineStr">
         <is>
-          <t>Chemo Do Brasil Comércio De Farmoquímicos Ltda</t>
+          <t>Shandong Anshun Pharmaceutical Co., Ltd.</t>
         </is>
       </c>
       <c r="B545" t="inlineStr">
         <is>
-          <t>drospirenona</t>
+          <t>tazobactam</t>
         </is>
       </c>
       <c r="C545" t="inlineStr">
         <is>
-          <t>25351273206202211</t>
+          <t>25351088152202291</t>
         </is>
       </c>
       <c r="D545" t="inlineStr">
         <is>
-          <t>005</t>
+          <t>001.1</t>
         </is>
       </c>
       <c r="E545" t="inlineStr">
         <is>
-          <t>23/05/2023</t>
+          <t>09/05/2023</t>
         </is>
       </c>
     </row>
     <row r="546">
       <c r="A546" t="inlineStr">
         <is>
-          <t>Shandong Anshun Pharmaceutical Co., Ltd.</t>
+          <t>Qilu Antibiotics Pharmaceutical Co., Ltd.</t>
         </is>
       </c>
       <c r="B546" t="inlineStr">
         <is>
-          <t>tazobactam</t>
+          <t>ceftriaxona dissódica hemieptaidratada</t>
         </is>
       </c>
       <c r="C546" t="inlineStr">
         <is>
-          <t>25351088152202291</t>
+          <t>25351535972202102</t>
         </is>
       </c>
       <c r="D546" t="inlineStr">
         <is>
-          <t>001.1</t>
+          <t>002.1</t>
         </is>
       </c>
       <c r="E546" t="inlineStr">
         <is>
-          <t>09/05/2023</t>
+          <t>08/05/2023</t>
         </is>
       </c>
     </row>
     <row r="547">
       <c r="A547" t="inlineStr">
         <is>
-          <t>Qilu Antibiotics Pharmaceutical Co., Ltd.</t>
+          <t>Antibióticos Do Brasil Ltda</t>
         </is>
       </c>
       <c r="B547" t="inlineStr">
         <is>
-          <t>ceftriaxona dissódica hemieptaidratada</t>
+          <t>ceftazidima pentaidratada</t>
         </is>
       </c>
       <c r="C547" t="inlineStr">
         <is>
-          <t>25351535972202102</t>
+          <t>25351063708202155</t>
         </is>
       </c>
       <c r="D547" t="inlineStr">
         <is>
-          <t>002.1</t>
+          <t>001</t>
         </is>
       </c>
       <c r="E547" t="inlineStr">
         <is>
-          <t>08/05/2023</t>
+          <t>02/05/2023</t>
         </is>
       </c>
     </row>
     <row r="548">
       <c r="A548" t="inlineStr">
         <is>
-          <t>Antibióticos Do Brasil Ltda</t>
+          <t>Farmson Basic Drugs Private Limited</t>
         </is>
       </c>
       <c r="B548" t="inlineStr">
         <is>
-          <t>ceftazidima pentaidratada</t>
+          <t>paracetamol</t>
         </is>
       </c>
       <c r="C548" t="inlineStr">
         <is>
-          <t>25351063708202155</t>
+          <t>25351898107202166</t>
         </is>
       </c>
       <c r="D548" t="inlineStr">
         <is>
-          <t>001</t>
+          <t>002</t>
         </is>
       </c>
       <c r="E548" t="inlineStr">
         <is>
-          <t>02/05/2023</t>
+          <t>27/04/2023</t>
         </is>
       </c>
     </row>
     <row r="549">
       <c r="A549" t="inlineStr">
         <is>
-          <t>Farmson Basic Drugs Private Limited</t>
+          <t>Alivus Life Sciences Limited</t>
         </is>
       </c>
       <c r="B549" t="inlineStr">
         <is>
-          <t>paracetamol</t>
+          <t>etoricoxibe</t>
         </is>
       </c>
       <c r="C549" t="inlineStr">
         <is>
-          <t>25351898107202166</t>
+          <t>25351514251202151</t>
         </is>
       </c>
       <c r="D549" t="inlineStr">
@@ -15235,51 +15235,51 @@
       </c>
       <c r="E549" t="inlineStr">
         <is>
-          <t>27/04/2023</t>
+          <t>26/04/2023</t>
         </is>
       </c>
     </row>
     <row r="550">
       <c r="A550" t="inlineStr">
         <is>
-          <t>Alivus Life Sciences Limited</t>
+          <t>Gland Pharma Limited</t>
         </is>
       </c>
       <c r="B550" t="inlineStr">
         <is>
-          <t>etoricoxibe</t>
+          <t>brometo de rocurônio</t>
         </is>
       </c>
       <c r="C550" t="inlineStr">
         <is>
-          <t>25351514251202151</t>
+          <t>25351037183202283</t>
         </is>
       </c>
       <c r="D550" t="inlineStr">
         <is>
-          <t>002</t>
+          <t>001</t>
         </is>
       </c>
       <c r="E550" t="inlineStr">
         <is>
-          <t>26/04/2023</t>
+          <t>18/04/2023</t>
         </is>
       </c>
     </row>
     <row r="551">
       <c r="A551" t="inlineStr">
         <is>
-          <t>Gland Pharma Limited</t>
+          <t>Intas Pharmaceuticals Limited</t>
         </is>
       </c>
       <c r="B551" t="inlineStr">
         <is>
-          <t>brometo de rocurônio</t>
+          <t>cloridrato de doxorrubicina</t>
         </is>
       </c>
       <c r="C551" t="inlineStr">
         <is>
-          <t>25351037183202283</t>
+          <t>25351604159202181</t>
         </is>
       </c>
       <c r="D551" t="inlineStr">
@@ -15296,17 +15296,17 @@
     <row r="552">
       <c r="A552" t="inlineStr">
         <is>
-          <t>Intas Pharmaceuticals Limited</t>
+          <t>Janssen-Cilag Farmaceutica Ltda</t>
         </is>
       </c>
       <c r="B552" t="inlineStr">
         <is>
-          <t>cloridrato de doxorrubicina</t>
+          <t>cloridrato de rilpivirina</t>
         </is>
       </c>
       <c r="C552" t="inlineStr">
         <is>
-          <t>25351604159202181</t>
+          <t>25351221052202100</t>
         </is>
       </c>
       <c r="D552" t="inlineStr">
@@ -15316,7 +15316,7 @@
       </c>
       <c r="E552" t="inlineStr">
         <is>
-          <t>18/04/2023</t>
+          <t>14/04/2023</t>
         </is>
       </c>
     </row>
@@ -15328,44 +15328,44 @@
       </c>
       <c r="B553" t="inlineStr">
         <is>
-          <t>cloridrato de rilpivirina</t>
+          <t>rilpivirina</t>
         </is>
       </c>
       <c r="C553" t="inlineStr">
         <is>
-          <t>25351221052202100</t>
+          <t>25351381305202195</t>
         </is>
       </c>
       <c r="D553" t="inlineStr">
         <is>
-          <t>001</t>
+          <t>002</t>
         </is>
       </c>
       <c r="E553" t="inlineStr">
         <is>
-          <t>14/04/2023</t>
+          <t>05/04/2023</t>
         </is>
       </c>
     </row>
     <row r="554">
       <c r="A554" t="inlineStr">
         <is>
-          <t>Janssen-Cilag Farmaceutica Ltda</t>
+          <t>Alembic Pharmaceuticals Limited</t>
         </is>
       </c>
       <c r="B554" t="inlineStr">
         <is>
-          <t>rilpivirina</t>
+          <t>etoricoxibe</t>
         </is>
       </c>
       <c r="C554" t="inlineStr">
         <is>
-          <t>25351381305202195</t>
+          <t>25351459577202116</t>
         </is>
       </c>
       <c r="D554" t="inlineStr">
         <is>
-          <t>002</t>
+          <t>001</t>
         </is>
       </c>
       <c r="E554" t="inlineStr">
@@ -15377,71 +15377,71 @@
     <row r="555">
       <c r="A555" t="inlineStr">
         <is>
-          <t>Alembic Pharmaceuticals Limited</t>
+          <t>Shandong Anshun Pharmaceutical Co., Ltd.</t>
         </is>
       </c>
       <c r="B555" t="inlineStr">
         <is>
-          <t>etoricoxibe</t>
+          <t>piperacilina monoidratada</t>
         </is>
       </c>
       <c r="C555" t="inlineStr">
         <is>
-          <t>25351459577202116</t>
+          <t>25351088151202246</t>
         </is>
       </c>
       <c r="D555" t="inlineStr">
         <is>
-          <t>001</t>
+          <t>001.1</t>
         </is>
       </c>
       <c r="E555" t="inlineStr">
         <is>
-          <t>05/04/2023</t>
+          <t>30/03/2023</t>
         </is>
       </c>
     </row>
     <row r="556">
       <c r="A556" t="inlineStr">
         <is>
-          <t>Shandong Anshun Pharmaceutical Co., Ltd.</t>
+          <t>Chemo Do Brasil Comércio De Farmoquímicos Ltda</t>
         </is>
       </c>
       <c r="B556" t="inlineStr">
         <is>
-          <t>piperacilina monoidratada</t>
+          <t>etinilestradiol</t>
         </is>
       </c>
       <c r="C556" t="inlineStr">
         <is>
-          <t>25351088151202246</t>
+          <t>25351788882202295</t>
         </is>
       </c>
       <c r="D556" t="inlineStr">
         <is>
-          <t>001.1</t>
+          <t>002</t>
         </is>
       </c>
       <c r="E556" t="inlineStr">
         <is>
-          <t>30/03/2023</t>
+          <t>23/03/2023</t>
         </is>
       </c>
     </row>
     <row r="557">
       <c r="A557" t="inlineStr">
         <is>
-          <t>Chemo Do Brasil Comércio De Farmoquímicos Ltda</t>
+          <t>Zhejiang Guobang Pharmaceutical Co., Ltd</t>
         </is>
       </c>
       <c r="B557" t="inlineStr">
         <is>
-          <t>etinilestradiol</t>
+          <t>azitromicina di-hidratada</t>
         </is>
       </c>
       <c r="C557" t="inlineStr">
         <is>
-          <t>25351788882202295</t>
+          <t>25351198490202159</t>
         </is>
       </c>
       <c r="D557" t="inlineStr">
@@ -15451,29 +15451,29 @@
       </c>
       <c r="E557" t="inlineStr">
         <is>
-          <t>23/03/2023</t>
+          <t>23/02/2023</t>
         </is>
       </c>
     </row>
     <row r="558">
       <c r="A558" t="inlineStr">
         <is>
-          <t>Zhejiang Guobang Pharmaceutical Co., Ltd</t>
+          <t>Intas Pharmaceuticals Limited</t>
         </is>
       </c>
       <c r="B558" t="inlineStr">
         <is>
-          <t>azitromicina di-hidratada</t>
+          <t>fampridina</t>
         </is>
       </c>
       <c r="C558" t="inlineStr">
         <is>
-          <t>25351198490202159</t>
+          <t>25351007864202217</t>
         </is>
       </c>
       <c r="D558" t="inlineStr">
         <is>
-          <t>002</t>
+          <t>001</t>
         </is>
       </c>
       <c r="E558" t="inlineStr">
@@ -15485,17 +15485,17 @@
     <row r="559">
       <c r="A559" t="inlineStr">
         <is>
-          <t>Intas Pharmaceuticals Limited</t>
+          <t>Hetero Labs Limited</t>
         </is>
       </c>
       <c r="B559" t="inlineStr">
         <is>
-          <t>fampridina</t>
+          <t>bicalutamida</t>
         </is>
       </c>
       <c r="C559" t="inlineStr">
         <is>
-          <t>25351007864202217</t>
+          <t>25351159727202003</t>
         </is>
       </c>
       <c r="D559" t="inlineStr">
@@ -15505,24 +15505,24 @@
       </c>
       <c r="E559" t="inlineStr">
         <is>
-          <t>23/02/2023</t>
+          <t>15/02/2023</t>
         </is>
       </c>
     </row>
     <row r="560">
       <c r="A560" t="inlineStr">
         <is>
-          <t>Hetero Labs Limited</t>
+          <t>Msn Laboratories Private Limited</t>
         </is>
       </c>
       <c r="B560" t="inlineStr">
         <is>
-          <t>bicalutamida</t>
+          <t>enzalutamida</t>
         </is>
       </c>
       <c r="C560" t="inlineStr">
         <is>
-          <t>25351159727202003</t>
+          <t>25351042982202191</t>
         </is>
       </c>
       <c r="D560" t="inlineStr">
@@ -15532,24 +15532,24 @@
       </c>
       <c r="E560" t="inlineStr">
         <is>
-          <t>15/02/2023</t>
+          <t>13/02/2023</t>
         </is>
       </c>
     </row>
     <row r="561">
       <c r="A561" t="inlineStr">
         <is>
-          <t>Msn Laboratories Private Limited</t>
+          <t>Fersinsa Gb S.A. De C.V.</t>
         </is>
       </c>
       <c r="B561" t="inlineStr">
         <is>
-          <t>enzalutamida</t>
+          <t>benzilpenicilina potássica</t>
         </is>
       </c>
       <c r="C561" t="inlineStr">
         <is>
-          <t>25351042982202191</t>
+          <t>25351881526202169</t>
         </is>
       </c>
       <c r="D561" t="inlineStr">
@@ -15559,24 +15559,24 @@
       </c>
       <c r="E561" t="inlineStr">
         <is>
-          <t>13/02/2023</t>
+          <t>01/02/2023</t>
         </is>
       </c>
     </row>
     <row r="562">
       <c r="A562" t="inlineStr">
         <is>
-          <t>Fersinsa Gb S.A. De C.V.</t>
+          <t>Transo-Pharm Handels-Gmbh</t>
         </is>
       </c>
       <c r="B562" t="inlineStr">
         <is>
-          <t>benzilpenicilina potássica</t>
+          <t>cloridrato de doxorrubicina</t>
         </is>
       </c>
       <c r="C562" t="inlineStr">
         <is>
-          <t>25351881526202169</t>
+          <t>25351666895202123</t>
         </is>
       </c>
       <c r="D562" t="inlineStr">
@@ -15593,17 +15593,17 @@
     <row r="563">
       <c r="A563" t="inlineStr">
         <is>
-          <t>Transo-Pharm Handels-Gmbh</t>
+          <t>Cyg Biotech Qumica &amp; Farmaceutica Ltda.</t>
         </is>
       </c>
       <c r="B563" t="inlineStr">
         <is>
-          <t>cloridrato de doxorrubicina</t>
+          <t>carbonato de lítio</t>
         </is>
       </c>
       <c r="C563" t="inlineStr">
         <is>
-          <t>25351666895202123</t>
+          <t>25351759475202190</t>
         </is>
       </c>
       <c r="D563" t="inlineStr">
@@ -15613,56 +15613,56 @@
       </c>
       <c r="E563" t="inlineStr">
         <is>
-          <t>01/02/2023</t>
+          <t>28/12/2022</t>
         </is>
       </c>
     </row>
     <row r="564">
       <c r="A564" t="inlineStr">
         <is>
-          <t>Cyg Biotech Qumica &amp; Farmaceutica Ltda.</t>
+          <t>Zhejiang Hisun Pharmaceutical Co., Ltd.</t>
         </is>
       </c>
       <c r="B564" t="inlineStr">
         <is>
-          <t>carbonato de lítio</t>
+          <t>tigeciclina</t>
         </is>
       </c>
       <c r="C564" t="inlineStr">
         <is>
-          <t>25351759475202190</t>
+          <t>25351970820202063</t>
         </is>
       </c>
       <c r="D564" t="inlineStr">
         <is>
-          <t>001</t>
+          <t>002</t>
         </is>
       </c>
       <c r="E564" t="inlineStr">
         <is>
-          <t>28/12/2022</t>
+          <t>07/12/2022</t>
         </is>
       </c>
     </row>
     <row r="565">
       <c r="A565" t="inlineStr">
         <is>
-          <t>Zhejiang Hisun Pharmaceutical Co., Ltd.</t>
+          <t>Alembic Pharmaceuticals Limited</t>
         </is>
       </c>
       <c r="B565" t="inlineStr">
         <is>
-          <t>tigeciclina</t>
+          <t>succinato de desvenlafaxina monoidratado</t>
         </is>
       </c>
       <c r="C565" t="inlineStr">
         <is>
-          <t>25351970820202063</t>
+          <t>25351114763202111</t>
         </is>
       </c>
       <c r="D565" t="inlineStr">
         <is>
-          <t>002</t>
+          <t>001.1</t>
         </is>
       </c>
       <c r="E565" t="inlineStr">
@@ -15674,27 +15674,27 @@
     <row r="566">
       <c r="A566" t="inlineStr">
         <is>
-          <t>Alembic Pharmaceuticals Limited</t>
+          <t>Msn Laboratories Private Limited</t>
         </is>
       </c>
       <c r="B566" t="inlineStr">
         <is>
-          <t>succinato de desvenlafaxina monoidratado</t>
+          <t>gefitinibe</t>
         </is>
       </c>
       <c r="C566" t="inlineStr">
         <is>
-          <t>25351114763202111</t>
+          <t>25351199392202139</t>
         </is>
       </c>
       <c r="D566" t="inlineStr">
         <is>
-          <t>001.1</t>
+          <t>001</t>
         </is>
       </c>
       <c r="E566" t="inlineStr">
         <is>
-          <t>07/12/2022</t>
+          <t>16/11/2022</t>
         </is>
       </c>
     </row>
@@ -15706,12 +15706,12 @@
       </c>
       <c r="B567" t="inlineStr">
         <is>
-          <t>gefitinibe</t>
+          <t>esilato de nintedanibe</t>
         </is>
       </c>
       <c r="C567" t="inlineStr">
         <is>
-          <t>25351199392202139</t>
+          <t>25351382611202068</t>
         </is>
       </c>
       <c r="D567" t="inlineStr">
@@ -15721,132 +15721,132 @@
       </c>
       <c r="E567" t="inlineStr">
         <is>
-          <t>16/11/2022</t>
+          <t>10/11/2022</t>
         </is>
       </c>
     </row>
     <row r="568">
       <c r="A568" t="inlineStr">
         <is>
-          <t>Msn Laboratories Private Limited</t>
+          <t>Harman Finochem Limited</t>
         </is>
       </c>
       <c r="B568" t="inlineStr">
         <is>
-          <t>esilato de nintedanibe</t>
+          <t>cloridrato de metformina</t>
         </is>
       </c>
       <c r="C568" t="inlineStr">
         <is>
-          <t>25351382611202068</t>
+          <t>25351223837202117</t>
         </is>
       </c>
       <c r="D568" t="inlineStr">
         <is>
-          <t>001</t>
+          <t>003</t>
         </is>
       </c>
       <c r="E568" t="inlineStr">
         <is>
-          <t>10/11/2022</t>
+          <t>25/10/2022</t>
         </is>
       </c>
     </row>
     <row r="569">
       <c r="A569" t="inlineStr">
         <is>
-          <t>Harman Finochem Limited</t>
+          <t>Biocon Limited</t>
         </is>
       </c>
       <c r="B569" t="inlineStr">
         <is>
-          <t>cloridrato de metformina</t>
+          <t>everolimo</t>
         </is>
       </c>
       <c r="C569" t="inlineStr">
         <is>
-          <t>25351223837202117</t>
+          <t>25351692063202162</t>
         </is>
       </c>
       <c r="D569" t="inlineStr">
         <is>
-          <t>003</t>
+          <t>002</t>
         </is>
       </c>
       <c r="E569" t="inlineStr">
         <is>
-          <t>25/10/2022</t>
+          <t>21/10/2022</t>
         </is>
       </c>
     </row>
     <row r="570">
       <c r="A570" t="inlineStr">
         <is>
-          <t>Biocon Limited</t>
+          <t>Synthimed Labs Private Limited</t>
         </is>
       </c>
       <c r="B570" t="inlineStr">
         <is>
-          <t>everolimo</t>
+          <t>claritromicina</t>
         </is>
       </c>
       <c r="C570" t="inlineStr">
         <is>
-          <t>25351692063202162</t>
+          <t>25351517246202281</t>
         </is>
       </c>
       <c r="D570" t="inlineStr">
         <is>
-          <t>002</t>
+          <t>003</t>
         </is>
       </c>
       <c r="E570" t="inlineStr">
         <is>
-          <t>21/10/2022</t>
+          <t>18/10/2022</t>
         </is>
       </c>
     </row>
     <row r="571">
       <c r="A571" t="inlineStr">
         <is>
-          <t>Synthimed Labs Private Limited</t>
+          <t>Shilpa Pharma Lifesciences Limited</t>
         </is>
       </c>
       <c r="B571" t="inlineStr">
         <is>
-          <t>claritromicina</t>
+          <t>cloridrato de bendamustina monoidratada</t>
         </is>
       </c>
       <c r="C571" t="inlineStr">
         <is>
-          <t>25351517246202281</t>
+          <t>25351748374202193</t>
         </is>
       </c>
       <c r="D571" t="inlineStr">
         <is>
-          <t>003</t>
+          <t>001</t>
         </is>
       </c>
       <c r="E571" t="inlineStr">
         <is>
-          <t>18/10/2022</t>
+          <t>14/10/2022</t>
         </is>
       </c>
     </row>
     <row r="572">
       <c r="A572" t="inlineStr">
         <is>
-          <t>Shilpa Pharma Lifesciences Limited</t>
+          <t>Msn Laboratories Private Limited</t>
         </is>
       </c>
       <c r="B572" t="inlineStr">
         <is>
-          <t>cloridrato de bendamustina monoidratada</t>
+          <t>tosilato de sorafenibe</t>
         </is>
       </c>
       <c r="C572" t="inlineStr">
         <is>
-          <t>25351748374202193</t>
+          <t>25351915465202141</t>
         </is>
       </c>
       <c r="D572" t="inlineStr">
@@ -15856,24 +15856,24 @@
       </c>
       <c r="E572" t="inlineStr">
         <is>
-          <t>14/10/2022</t>
+          <t>11/10/2022</t>
         </is>
       </c>
     </row>
     <row r="573">
       <c r="A573" t="inlineStr">
         <is>
-          <t>Msn Laboratories Private Limited</t>
+          <t>Sun Pharmaceutical Industries Limited</t>
         </is>
       </c>
       <c r="B573" t="inlineStr">
         <is>
-          <t>tosilato de sorafenibe</t>
+          <t>vildagliptina</t>
         </is>
       </c>
       <c r="C573" t="inlineStr">
         <is>
-          <t>25351915465202141</t>
+          <t>25351063743202255</t>
         </is>
       </c>
       <c r="D573" t="inlineStr">
@@ -15883,132 +15883,132 @@
       </c>
       <c r="E573" t="inlineStr">
         <is>
-          <t>11/10/2022</t>
+          <t>10/10/2022</t>
         </is>
       </c>
     </row>
     <row r="574">
       <c r="A574" t="inlineStr">
         <is>
-          <t>Sun Pharmaceutical Industries Limited</t>
+          <t>Zhejiang Charioteer Pharmaceutical Co., Ltd.</t>
         </is>
       </c>
       <c r="B574" t="inlineStr">
         <is>
-          <t>vildagliptina</t>
+          <t>aciclovir</t>
         </is>
       </c>
       <c r="C574" t="inlineStr">
         <is>
-          <t>25351063743202255</t>
+          <t>25351308050202116</t>
         </is>
       </c>
       <c r="D574" t="inlineStr">
         <is>
-          <t>001</t>
+          <t>002.1</t>
         </is>
       </c>
       <c r="E574" t="inlineStr">
         <is>
-          <t>10/10/2022</t>
+          <t>12/09/2022</t>
         </is>
       </c>
     </row>
     <row r="575">
       <c r="A575" t="inlineStr">
         <is>
-          <t>Zhejiang Charioteer Pharmaceutical Co., Ltd.</t>
+          <t>Shilpa Pharma Lifesciences Limited</t>
         </is>
       </c>
       <c r="B575" t="inlineStr">
         <is>
-          <t>aciclovir</t>
+          <t>bussulfano</t>
         </is>
       </c>
       <c r="C575" t="inlineStr">
         <is>
-          <t>25351308050202116</t>
+          <t>25351653813202181</t>
         </is>
       </c>
       <c r="D575" t="inlineStr">
         <is>
-          <t>002.1</t>
+          <t>002</t>
         </is>
       </c>
       <c r="E575" t="inlineStr">
         <is>
-          <t>12/09/2022</t>
+          <t>20/08/2022</t>
         </is>
       </c>
     </row>
     <row r="576">
       <c r="A576" t="inlineStr">
         <is>
-          <t>Shilpa Pharma Lifesciences Limited</t>
+          <t>Honour Lab Limited</t>
         </is>
       </c>
       <c r="B576" t="inlineStr">
         <is>
-          <t>bussulfano</t>
+          <t>fosfato de sitagliptina</t>
         </is>
       </c>
       <c r="C576" t="inlineStr">
         <is>
-          <t>25351653813202181</t>
+          <t>25351333869202031</t>
         </is>
       </c>
       <c r="D576" t="inlineStr">
         <is>
-          <t>002</t>
+          <t>001</t>
         </is>
       </c>
       <c r="E576" t="inlineStr">
         <is>
-          <t>20/08/2022</t>
+          <t>16/08/2022</t>
         </is>
       </c>
     </row>
     <row r="577">
       <c r="A577" t="inlineStr">
         <is>
-          <t>Honour Lab Limited</t>
+          <t>Fersinsa Gb S.A. De C.V.</t>
         </is>
       </c>
       <c r="B577" t="inlineStr">
         <is>
-          <t>fosfato de sitagliptina</t>
+          <t>amoxicilina tri-hidratada</t>
         </is>
       </c>
       <c r="C577" t="inlineStr">
         <is>
-          <t>25351333869202031</t>
+          <t>25351533263202001</t>
         </is>
       </c>
       <c r="D577" t="inlineStr">
         <is>
-          <t>001</t>
+          <t>002</t>
         </is>
       </c>
       <c r="E577" t="inlineStr">
         <is>
-          <t>16/08/2022</t>
+          <t>08/08/2022</t>
         </is>
       </c>
     </row>
     <row r="578">
       <c r="A578" t="inlineStr">
         <is>
-          <t>Fersinsa Gb S.A. De C.V.</t>
+          <t>Tapi Brazil Ltda</t>
         </is>
       </c>
       <c r="B578" t="inlineStr">
         <is>
-          <t>amoxicilina tri-hidratada</t>
+          <t>cloridrato de memantina</t>
         </is>
       </c>
       <c r="C578" t="inlineStr">
         <is>
-          <t>25351533263202001</t>
+          <t>25351537007202166</t>
         </is>
       </c>
       <c r="D578" t="inlineStr">
@@ -16018,51 +16018,51 @@
       </c>
       <c r="E578" t="inlineStr">
         <is>
-          <t>08/08/2022</t>
+          <t>18/07/2022</t>
         </is>
       </c>
     </row>
     <row r="579">
       <c r="A579" t="inlineStr">
         <is>
-          <t>Tapi Brazil Ltda</t>
+          <t>Alembic Pharmaceuticals Limited</t>
         </is>
       </c>
       <c r="B579" t="inlineStr">
         <is>
-          <t>cloridrato de memantina</t>
+          <t>vildagliptina</t>
         </is>
       </c>
       <c r="C579" t="inlineStr">
         <is>
-          <t>25351537007202166</t>
+          <t>25351871278202067</t>
         </is>
       </c>
       <c r="D579" t="inlineStr">
         <is>
-          <t>002</t>
+          <t>001</t>
         </is>
       </c>
       <c r="E579" t="inlineStr">
         <is>
-          <t>18/07/2022</t>
+          <t>04/04/2022</t>
         </is>
       </c>
     </row>
     <row r="580">
       <c r="A580" t="inlineStr">
         <is>
-          <t>Alembic Pharmaceuticals Limited</t>
+          <t>Msn Laboratories Private Limited</t>
         </is>
       </c>
       <c r="B580" t="inlineStr">
         <is>
-          <t>vildagliptina</t>
+          <t>rosuvastatina cálcica</t>
         </is>
       </c>
       <c r="C580" t="inlineStr">
         <is>
-          <t>25351871278202067</t>
+          <t>25351322289202018</t>
         </is>
       </c>
       <c r="D580" t="inlineStr">
@@ -16072,59 +16072,32 @@
       </c>
       <c r="E580" t="inlineStr">
         <is>
-          <t>04/04/2022</t>
+          <t>16/03/2022</t>
         </is>
       </c>
     </row>
     <row r="581">
       <c r="A581" t="inlineStr">
         <is>
-          <t>Msn Laboratories Private Limited</t>
+          <t>Viyash Scientific Limited</t>
         </is>
       </c>
       <c r="B581" t="inlineStr">
         <is>
-          <t>rosuvastatina cálcica</t>
+          <t>cloridrato  de ondansetrona di-hidratado</t>
         </is>
       </c>
       <c r="C581" t="inlineStr">
         <is>
-          <t>25351322289202018</t>
+          <t>25351163773202180</t>
         </is>
       </c>
       <c r="D581" t="inlineStr">
         <is>
-          <t>001</t>
+          <t>001.1</t>
         </is>
       </c>
       <c r="E581" t="inlineStr">
-        <is>
-          <t>16/03/2022</t>
-        </is>
-      </c>
-    </row>
-    <row r="582">
-      <c r="A582" t="inlineStr">
-        <is>
-          <t>Viyash Scientific Limited</t>
-        </is>
-      </c>
-      <c r="B582" t="inlineStr">
-        <is>
-          <t>cloridrato  de ondansetrona di-hidratado</t>
-        </is>
-      </c>
-      <c r="C582" t="inlineStr">
-        <is>
-          <t>25351163773202180</t>
-        </is>
-      </c>
-      <c r="D582" t="inlineStr">
-        <is>
-          <t>001.1</t>
-        </is>
-      </c>
-      <c r="E582" t="inlineStr">
         <is>
           <t>23/02/2022</t>
         </is>

</xml_diff>

<commit_message>
Atualiza lista de CADIFAs deferidas (execução automática 11/08/2026)
2 novas linhas: Abbvie Farmacêutica Ltda. (atogepanto hidratado, CADIFA 25351423937202303, Revisão 001.1) e Synthon Bv (sugamadex sódico, CADIFA 25351779849202193, Revisão 002).
</commit_message>
<xml_diff>
--- a/cadifa_completo.xlsx
+++ b/cadifa_completo.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E581"/>
+  <dimension ref="A1:E582"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -667,7 +667,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>atogepanto</t>
+          <t>atogepanto hidratado</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -677,7 +677,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>001</t>
+          <t>001.1</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -3524,7 +3524,7 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>Ind-Swift Laboratories Limited</t>
+          <t>Synthimed Labs Private Limited</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
@@ -5090,7 +5090,7 @@
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>Ind-Swift Laboratories Limited</t>
+          <t>Synthimed Labs Private Limited</t>
         </is>
       </c>
       <c r="B174" t="inlineStr">
@@ -13892,71 +13892,71 @@
     <row r="500">
       <c r="A500" t="inlineStr">
         <is>
-          <t>Fdc Limited</t>
+          <t>Synthon Bv</t>
         </is>
       </c>
       <c r="B500" t="inlineStr">
         <is>
-          <t>maleato de timolol</t>
+          <t>sugamadex sódico</t>
         </is>
       </c>
       <c r="C500" t="inlineStr">
         <is>
-          <t>25351087503202246</t>
+          <t>25351779849202193</t>
         </is>
       </c>
       <c r="D500" t="inlineStr">
         <is>
-          <t>001</t>
+          <t>002</t>
         </is>
       </c>
       <c r="E500" t="inlineStr">
         <is>
-          <t>09/11/2023</t>
+          <t>13/11/2023</t>
         </is>
       </c>
     </row>
     <row r="501">
       <c r="A501" t="inlineStr">
         <is>
-          <t>Medichem S.A.</t>
+          <t>Fdc Limited</t>
         </is>
       </c>
       <c r="B501" t="inlineStr">
         <is>
-          <t>micafungina sódica</t>
+          <t>maleato de timolol</t>
         </is>
       </c>
       <c r="C501" t="inlineStr">
         <is>
-          <t>25351543525202208</t>
+          <t>25351087503202246</t>
         </is>
       </c>
       <c r="D501" t="inlineStr">
         <is>
-          <t>002</t>
+          <t>001</t>
         </is>
       </c>
       <c r="E501" t="inlineStr">
         <is>
-          <t>06/11/2023</t>
+          <t>09/11/2023</t>
         </is>
       </c>
     </row>
     <row r="502">
       <c r="A502" t="inlineStr">
         <is>
-          <t>Harman Finochem Limited</t>
+          <t>Medichem S.A.</t>
         </is>
       </c>
       <c r="B502" t="inlineStr">
         <is>
-          <t>fenitoína</t>
+          <t>micafungina sódica</t>
         </is>
       </c>
       <c r="C502" t="inlineStr">
         <is>
-          <t>25351122886202214</t>
+          <t>25351543525202208</t>
         </is>
       </c>
       <c r="D502" t="inlineStr">
@@ -13966,24 +13966,24 @@
       </c>
       <c r="E502" t="inlineStr">
         <is>
-          <t>03/11/2023</t>
+          <t>06/11/2023</t>
         </is>
       </c>
     </row>
     <row r="503">
       <c r="A503" t="inlineStr">
         <is>
-          <t>Nortec Química S.A</t>
+          <t>Harman Finochem Limited</t>
         </is>
       </c>
       <c r="B503" t="inlineStr">
         <is>
-          <t>micofenolato de sódio</t>
+          <t>fenitoína</t>
         </is>
       </c>
       <c r="C503" t="inlineStr">
         <is>
-          <t>25351448083202289</t>
+          <t>25351122886202214</t>
         </is>
       </c>
       <c r="D503" t="inlineStr">
@@ -14000,49 +14000,49 @@
     <row r="504">
       <c r="A504" t="inlineStr">
         <is>
-          <t>Emcure Pharmaceuticals Limited</t>
+          <t>Nortec Química S.A</t>
         </is>
       </c>
       <c r="B504" t="inlineStr">
         <is>
-          <t>milrinona</t>
+          <t>micofenolato de sódio</t>
         </is>
       </c>
       <c r="C504" t="inlineStr">
         <is>
-          <t>25351038756202296</t>
+          <t>25351448083202289</t>
         </is>
       </c>
       <c r="D504" t="inlineStr">
         <is>
-          <t>001</t>
+          <t>002</t>
         </is>
       </c>
       <c r="E504" t="inlineStr">
         <is>
-          <t>30/10/2023</t>
+          <t>03/11/2023</t>
         </is>
       </c>
     </row>
     <row r="505">
       <c r="A505" t="inlineStr">
         <is>
-          <t>Neuland Laboratories Limited</t>
+          <t>Emcure Pharmaceuticals Limited</t>
         </is>
       </c>
       <c r="B505" t="inlineStr">
         <is>
-          <t>mirtazapina</t>
+          <t>milrinona</t>
         </is>
       </c>
       <c r="C505" t="inlineStr">
         <is>
-          <t>25351589465202261</t>
+          <t>25351038756202296</t>
         </is>
       </c>
       <c r="D505" t="inlineStr">
         <is>
-          <t>003</t>
+          <t>001</t>
         </is>
       </c>
       <c r="E505" t="inlineStr">
@@ -14054,44 +14054,44 @@
     <row r="506">
       <c r="A506" t="inlineStr">
         <is>
-          <t>Ctx Lifesciences Pvt. Ltd.</t>
+          <t>Neuland Laboratories Limited</t>
         </is>
       </c>
       <c r="B506" t="inlineStr">
         <is>
-          <t>succinato de metoprolol</t>
+          <t>mirtazapina</t>
         </is>
       </c>
       <c r="C506" t="inlineStr">
         <is>
-          <t>25351287504202116</t>
+          <t>25351589465202261</t>
         </is>
       </c>
       <c r="D506" t="inlineStr">
         <is>
-          <t>001</t>
+          <t>003</t>
         </is>
       </c>
       <c r="E506" t="inlineStr">
         <is>
-          <t>27/10/2023</t>
+          <t>30/10/2023</t>
         </is>
       </c>
     </row>
     <row r="507">
       <c r="A507" t="inlineStr">
         <is>
-          <t>Ulkar Kimya Sanayii Ve Ticaret A.S.</t>
+          <t>Ctx Lifesciences Pvt. Ltd.</t>
         </is>
       </c>
       <c r="B507" t="inlineStr">
         <is>
-          <t>etodolaco</t>
+          <t>succinato de metoprolol</t>
         </is>
       </c>
       <c r="C507" t="inlineStr">
         <is>
-          <t>25351171112202217</t>
+          <t>25351287504202116</t>
         </is>
       </c>
       <c r="D507" t="inlineStr">
@@ -14101,29 +14101,29 @@
       </c>
       <c r="E507" t="inlineStr">
         <is>
-          <t>25/10/2023</t>
+          <t>27/10/2023</t>
         </is>
       </c>
     </row>
     <row r="508">
       <c r="A508" t="inlineStr">
         <is>
-          <t>Msn Pharmachem Private Limited</t>
+          <t>Ulkar Kimya Sanayii Ve Ticaret A.S.</t>
         </is>
       </c>
       <c r="B508" t="inlineStr">
         <is>
-          <t>vildagliptina</t>
+          <t>etodolaco</t>
         </is>
       </c>
       <c r="C508" t="inlineStr">
         <is>
-          <t>25351407050202289</t>
+          <t>25351171112202217</t>
         </is>
       </c>
       <c r="D508" t="inlineStr">
         <is>
-          <t>002</t>
+          <t>001</t>
         </is>
       </c>
       <c r="E508" t="inlineStr">
@@ -14135,22 +14135,22 @@
     <row r="509">
       <c r="A509" t="inlineStr">
         <is>
-          <t>Cohance Lifesciences Limited</t>
+          <t>Msn Pharmachem Private Limited</t>
         </is>
       </c>
       <c r="B509" t="inlineStr">
         <is>
-          <t>lamotrigina</t>
+          <t>vildagliptina</t>
         </is>
       </c>
       <c r="C509" t="inlineStr">
         <is>
-          <t>25351699210202125</t>
+          <t>25351407050202289</t>
         </is>
       </c>
       <c r="D509" t="inlineStr">
         <is>
-          <t>001</t>
+          <t>002</t>
         </is>
       </c>
       <c r="E509" t="inlineStr">
@@ -14162,17 +14162,17 @@
     <row r="510">
       <c r="A510" t="inlineStr">
         <is>
-          <t>Hubei Yitai Pharmaceutical Co., Ltd.</t>
+          <t>Cohance Lifesciences Limited</t>
         </is>
       </c>
       <c r="B510" t="inlineStr">
         <is>
-          <t>aciclovir</t>
+          <t>lamotrigina</t>
         </is>
       </c>
       <c r="C510" t="inlineStr">
         <is>
-          <t>25351473051202131</t>
+          <t>25351699210202125</t>
         </is>
       </c>
       <c r="D510" t="inlineStr">
@@ -14182,29 +14182,29 @@
       </c>
       <c r="E510" t="inlineStr">
         <is>
-          <t>24/10/2023</t>
+          <t>25/10/2023</t>
         </is>
       </c>
     </row>
     <row r="511">
       <c r="A511" t="inlineStr">
         <is>
-          <t>Janssen-Cilag Farmaceutica Ltda</t>
+          <t>Hubei Yitai Pharmaceutical Co., Ltd.</t>
         </is>
       </c>
       <c r="B511" t="inlineStr">
         <is>
-          <t>etanolato de darunavir</t>
+          <t>aciclovir</t>
         </is>
       </c>
       <c r="C511" t="inlineStr">
         <is>
-          <t>25351122285202201</t>
+          <t>25351473051202131</t>
         </is>
       </c>
       <c r="D511" t="inlineStr">
         <is>
-          <t>002</t>
+          <t>001</t>
         </is>
       </c>
       <c r="E511" t="inlineStr">
@@ -14216,17 +14216,17 @@
     <row r="512">
       <c r="A512" t="inlineStr">
         <is>
-          <t>Torrent Pharmaceuticals Limited</t>
+          <t>Janssen-Cilag Farmaceutica Ltda</t>
         </is>
       </c>
       <c r="B512" t="inlineStr">
         <is>
-          <t>lamotrigina</t>
+          <t>etanolato de darunavir</t>
         </is>
       </c>
       <c r="C512" t="inlineStr">
         <is>
-          <t>25351171478202288</t>
+          <t>25351122285202201</t>
         </is>
       </c>
       <c r="D512" t="inlineStr">
@@ -14236,56 +14236,56 @@
       </c>
       <c r="E512" t="inlineStr">
         <is>
-          <t>23/10/2023</t>
+          <t>24/10/2023</t>
         </is>
       </c>
     </row>
     <row r="513">
       <c r="A513" t="inlineStr">
         <is>
-          <t>Wuhan Wuyao Pharmaceutical Co., Ltd.</t>
+          <t>Torrent Pharmaceuticals Limited</t>
         </is>
       </c>
       <c r="B513" t="inlineStr">
         <is>
-          <t>dipirona monoidratada</t>
+          <t>lamotrigina</t>
         </is>
       </c>
       <c r="C513" t="inlineStr">
         <is>
-          <t>25351596512202223</t>
+          <t>25351171478202288</t>
         </is>
       </c>
       <c r="D513" t="inlineStr">
         <is>
-          <t>001</t>
+          <t>002</t>
         </is>
       </c>
       <c r="E513" t="inlineStr">
         <is>
-          <t>11/10/2023</t>
+          <t>23/10/2023</t>
         </is>
       </c>
     </row>
     <row r="514">
       <c r="A514" t="inlineStr">
         <is>
-          <t>Tapi Brazil Ltda</t>
+          <t>Wuhan Wuyao Pharmaceutical Co., Ltd.</t>
         </is>
       </c>
       <c r="B514" t="inlineStr">
         <is>
-          <t>dasatinibe monoidratado</t>
+          <t>dipirona monoidratada</t>
         </is>
       </c>
       <c r="C514" t="inlineStr">
         <is>
-          <t>25351543510202231</t>
+          <t>25351596512202223</t>
         </is>
       </c>
       <c r="D514" t="inlineStr">
         <is>
-          <t>002.1</t>
+          <t>001</t>
         </is>
       </c>
       <c r="E514" t="inlineStr">
@@ -14297,44 +14297,44 @@
     <row r="515">
       <c r="A515" t="inlineStr">
         <is>
-          <t>Sun Pharmaceutical Industries Limited</t>
+          <t>Tapi Brazil Ltda</t>
         </is>
       </c>
       <c r="B515" t="inlineStr">
         <is>
-          <t>cloridrato de donepezila monoidratado</t>
+          <t>dasatinibe monoidratado</t>
         </is>
       </c>
       <c r="C515" t="inlineStr">
         <is>
-          <t>25351244345202238</t>
+          <t>25351543510202231</t>
         </is>
       </c>
       <c r="D515" t="inlineStr">
         <is>
-          <t>001</t>
+          <t>002.1</t>
         </is>
       </c>
       <c r="E515" t="inlineStr">
         <is>
-          <t>05/10/2023</t>
+          <t>11/10/2023</t>
         </is>
       </c>
     </row>
     <row r="516">
       <c r="A516" t="inlineStr">
         <is>
-          <t>Zhejiang Hisun Pharmaceutical Co., Ltd.</t>
+          <t>Sun Pharmaceutical Industries Limited</t>
         </is>
       </c>
       <c r="B516" t="inlineStr">
         <is>
-          <t>adenosina</t>
+          <t>cloridrato de donepezila monoidratado</t>
         </is>
       </c>
       <c r="C516" t="inlineStr">
         <is>
-          <t>25351008874202199</t>
+          <t>25351244345202238</t>
         </is>
       </c>
       <c r="D516" t="inlineStr">
@@ -14344,29 +14344,29 @@
       </c>
       <c r="E516" t="inlineStr">
         <is>
-          <t>03/10/2023</t>
+          <t>05/10/2023</t>
         </is>
       </c>
     </row>
     <row r="517">
       <c r="A517" t="inlineStr">
         <is>
-          <t>Moehs Ibérica, S.L.</t>
+          <t>Zhejiang Hisun Pharmaceutical Co., Ltd.</t>
         </is>
       </c>
       <c r="B517" t="inlineStr">
         <is>
-          <t>hemifumarato de bisoprolol</t>
+          <t>adenosina</t>
         </is>
       </c>
       <c r="C517" t="inlineStr">
         <is>
-          <t>25351618932202197</t>
+          <t>25351008874202199</t>
         </is>
       </c>
       <c r="D517" t="inlineStr">
         <is>
-          <t>002.1</t>
+          <t>001</t>
         </is>
       </c>
       <c r="E517" t="inlineStr">
@@ -14378,49 +14378,49 @@
     <row r="518">
       <c r="A518" t="inlineStr">
         <is>
-          <t>Tapi Brazil Ltda</t>
+          <t>Moehs Ibérica, S.L.</t>
         </is>
       </c>
       <c r="B518" t="inlineStr">
         <is>
-          <t>rivaroxabana</t>
+          <t>hemifumarato de bisoprolol</t>
         </is>
       </c>
       <c r="C518" t="inlineStr">
         <is>
-          <t>25351312133202291</t>
+          <t>25351618932202197</t>
         </is>
       </c>
       <c r="D518" t="inlineStr">
         <is>
-          <t>003</t>
+          <t>002.1</t>
         </is>
       </c>
       <c r="E518" t="inlineStr">
         <is>
-          <t>26/09/2023</t>
+          <t>03/10/2023</t>
         </is>
       </c>
     </row>
     <row r="519">
       <c r="A519" t="inlineStr">
         <is>
-          <t>Shilpa Pharma Lifesciences Limited</t>
+          <t>Tapi Brazil Ltda</t>
         </is>
       </c>
       <c r="B519" t="inlineStr">
         <is>
-          <t>bortezomibe</t>
+          <t>rivaroxabana</t>
         </is>
       </c>
       <c r="C519" t="inlineStr">
         <is>
-          <t>25351839141202107</t>
+          <t>25351312133202291</t>
         </is>
       </c>
       <c r="D519" t="inlineStr">
         <is>
-          <t>001</t>
+          <t>003</t>
         </is>
       </c>
       <c r="E519" t="inlineStr">
@@ -14432,22 +14432,22 @@
     <row r="520">
       <c r="A520" t="inlineStr">
         <is>
-          <t>Dr Reddys Farmacêutica Do Brasil Ltda</t>
+          <t>Shilpa Pharma Lifesciences Limited</t>
         </is>
       </c>
       <c r="B520" t="inlineStr">
         <is>
-          <t>lenalidomida</t>
+          <t>bortezomibe</t>
         </is>
       </c>
       <c r="C520" t="inlineStr">
         <is>
-          <t>25351068660202252</t>
+          <t>25351839141202107</t>
         </is>
       </c>
       <c r="D520" t="inlineStr">
         <is>
-          <t>003</t>
+          <t>001</t>
         </is>
       </c>
       <c r="E520" t="inlineStr">
@@ -14459,49 +14459,49 @@
     <row r="521">
       <c r="A521" t="inlineStr">
         <is>
-          <t>Zhuhai United Laboratories Co., Ltd.</t>
+          <t>Dr Reddys Farmacêutica Do Brasil Ltda</t>
         </is>
       </c>
       <c r="B521" t="inlineStr">
         <is>
-          <t>ampicilina sódica</t>
+          <t>lenalidomida</t>
         </is>
       </c>
       <c r="C521" t="inlineStr">
         <is>
-          <t>25351433410202117</t>
+          <t>25351068660202252</t>
         </is>
       </c>
       <c r="D521" t="inlineStr">
         <is>
-          <t>002.1</t>
+          <t>003</t>
         </is>
       </c>
       <c r="E521" t="inlineStr">
         <is>
-          <t>22/09/2023</t>
+          <t>26/09/2023</t>
         </is>
       </c>
     </row>
     <row r="522">
       <c r="A522" t="inlineStr">
         <is>
-          <t>Chemwerth, Inc.</t>
+          <t>Zhuhai United Laboratories Co., Ltd.</t>
         </is>
       </c>
       <c r="B522" t="inlineStr">
         <is>
-          <t>milrinona</t>
+          <t>ampicilina sódica</t>
         </is>
       </c>
       <c r="C522" t="inlineStr">
         <is>
-          <t>25351869642202118</t>
+          <t>25351433410202117</t>
         </is>
       </c>
       <c r="D522" t="inlineStr">
         <is>
-          <t>001.1</t>
+          <t>002.1</t>
         </is>
       </c>
       <c r="E522" t="inlineStr">
@@ -14513,17 +14513,17 @@
     <row r="523">
       <c r="A523" t="inlineStr">
         <is>
-          <t>Msn Pharmachem Private Limited</t>
+          <t>Chemwerth, Inc.</t>
         </is>
       </c>
       <c r="B523" t="inlineStr">
         <is>
-          <t>bromidrato de vortioxetina</t>
+          <t>milrinona</t>
         </is>
       </c>
       <c r="C523" t="inlineStr">
         <is>
-          <t>25351252213202280</t>
+          <t>25351869642202118</t>
         </is>
       </c>
       <c r="D523" t="inlineStr">
@@ -14533,83 +14533,83 @@
       </c>
       <c r="E523" t="inlineStr">
         <is>
-          <t>18/09/2023</t>
+          <t>22/09/2023</t>
         </is>
       </c>
     </row>
     <row r="524">
       <c r="A524" t="inlineStr">
         <is>
-          <t>Matrix Pharmacorp Private Limited</t>
+          <t>Msn Pharmachem Private Limited</t>
         </is>
       </c>
       <c r="B524" t="inlineStr">
         <is>
-          <t>hemitartarato de zolpidem</t>
+          <t>bromidrato de vortioxetina</t>
         </is>
       </c>
       <c r="C524" t="inlineStr">
         <is>
-          <t>25351580744202189</t>
+          <t>25351252213202280</t>
         </is>
       </c>
       <c r="D524" t="inlineStr">
         <is>
-          <t>003</t>
+          <t>001.1</t>
         </is>
       </c>
       <c r="E524" t="inlineStr">
         <is>
-          <t>08/09/2023</t>
+          <t>18/09/2023</t>
         </is>
       </c>
     </row>
     <row r="525">
       <c r="A525" t="inlineStr">
         <is>
-          <t>Msn Pharmachem Private Limited</t>
+          <t>Matrix Pharmacorp Private Limited</t>
         </is>
       </c>
       <c r="B525" t="inlineStr">
         <is>
-          <t>aripiprazol</t>
+          <t>hemitartarato de zolpidem</t>
         </is>
       </c>
       <c r="C525" t="inlineStr">
         <is>
-          <t>25351524957202210</t>
+          <t>25351580744202189</t>
         </is>
       </c>
       <c r="D525" t="inlineStr">
         <is>
-          <t>002</t>
+          <t>003</t>
         </is>
       </c>
       <c r="E525" t="inlineStr">
         <is>
-          <t>05/09/2023</t>
+          <t>08/09/2023</t>
         </is>
       </c>
     </row>
     <row r="526">
       <c r="A526" t="inlineStr">
         <is>
-          <t>Sun Pharmaceutical Industries Limited</t>
+          <t>Msn Pharmachem Private Limited</t>
         </is>
       </c>
       <c r="B526" t="inlineStr">
         <is>
-          <t>mesilato de lenvatinibe</t>
+          <t>aripiprazol</t>
         </is>
       </c>
       <c r="C526" t="inlineStr">
         <is>
-          <t>25351206913202201</t>
+          <t>25351524957202210</t>
         </is>
       </c>
       <c r="D526" t="inlineStr">
         <is>
-          <t>001</t>
+          <t>002</t>
         </is>
       </c>
       <c r="E526" t="inlineStr">
@@ -14621,17 +14621,17 @@
     <row r="527">
       <c r="A527" t="inlineStr">
         <is>
-          <t>Dr Reddys Farmacêutica Do Brasil Ltda</t>
+          <t>Sun Pharmaceutical Industries Limited</t>
         </is>
       </c>
       <c r="B527" t="inlineStr">
         <is>
-          <t>cloridrato de naratriptana</t>
+          <t>mesilato de lenvatinibe</t>
         </is>
       </c>
       <c r="C527" t="inlineStr">
         <is>
-          <t>25351673613202225</t>
+          <t>25351206913202201</t>
         </is>
       </c>
       <c r="D527" t="inlineStr">
@@ -14648,17 +14648,17 @@
     <row r="528">
       <c r="A528" t="inlineStr">
         <is>
-          <t>Intas Pharmaceuticals Limited</t>
+          <t>Dr Reddys Farmacêutica Do Brasil Ltda</t>
         </is>
       </c>
       <c r="B528" t="inlineStr">
         <is>
-          <t>carfilzomibe</t>
+          <t>cloridrato de naratriptana</t>
         </is>
       </c>
       <c r="C528" t="inlineStr">
         <is>
-          <t>25351255810202185</t>
+          <t>25351673613202225</t>
         </is>
       </c>
       <c r="D528" t="inlineStr">
@@ -14668,78 +14668,78 @@
       </c>
       <c r="E528" t="inlineStr">
         <is>
-          <t>31/08/2023</t>
+          <t>05/09/2023</t>
         </is>
       </c>
     </row>
     <row r="529">
       <c r="A529" t="inlineStr">
         <is>
-          <t>Scl Lifesciences Limited</t>
+          <t>Intas Pharmaceuticals Limited</t>
         </is>
       </c>
       <c r="B529" t="inlineStr">
         <is>
-          <t>trometamol cetorolaco</t>
+          <t>carfilzomibe</t>
         </is>
       </c>
       <c r="C529" t="inlineStr">
         <is>
-          <t>25351654225202164</t>
+          <t>25351255810202185</t>
         </is>
       </c>
       <c r="D529" t="inlineStr">
         <is>
-          <t>002</t>
+          <t>001</t>
         </is>
       </c>
       <c r="E529" t="inlineStr">
         <is>
-          <t>29/08/2023</t>
+          <t>31/08/2023</t>
         </is>
       </c>
     </row>
     <row r="530">
       <c r="A530" t="inlineStr">
         <is>
-          <t>Msn Laboratories Private Limited</t>
+          <t>Scl Lifesciences Limited</t>
         </is>
       </c>
       <c r="B530" t="inlineStr">
         <is>
-          <t>pitavastatina cálcica pentaidratada</t>
+          <t>trometamol cetorolaco</t>
         </is>
       </c>
       <c r="C530" t="inlineStr">
         <is>
-          <t>25351527145202218</t>
+          <t>25351654225202164</t>
         </is>
       </c>
       <c r="D530" t="inlineStr">
         <is>
-          <t>001</t>
+          <t>002</t>
         </is>
       </c>
       <c r="E530" t="inlineStr">
         <is>
-          <t>28/08/2023</t>
+          <t>29/08/2023</t>
         </is>
       </c>
     </row>
     <row r="531">
       <c r="A531" t="inlineStr">
         <is>
-          <t>Glochem Industries Private Limited</t>
+          <t>Msn Laboratories Private Limited</t>
         </is>
       </c>
       <c r="B531" t="inlineStr">
         <is>
-          <t>besilato de levanlodipino hemipentaidratado</t>
+          <t>pitavastatina cálcica pentaidratada</t>
         </is>
       </c>
       <c r="C531" t="inlineStr">
         <is>
-          <t>25351492777202253</t>
+          <t>25351527145202218</t>
         </is>
       </c>
       <c r="D531" t="inlineStr">
@@ -14749,24 +14749,24 @@
       </c>
       <c r="E531" t="inlineStr">
         <is>
-          <t>23/08/2023</t>
+          <t>28/08/2023</t>
         </is>
       </c>
     </row>
     <row r="532">
       <c r="A532" t="inlineStr">
         <is>
-          <t>Ipca Laboratories Ltd.</t>
+          <t>Glochem Industries Private Limited</t>
         </is>
       </c>
       <c r="B532" t="inlineStr">
         <is>
-          <t>hidroclorotiazida</t>
+          <t>besilato de levanlodipino hemipentaidratado</t>
         </is>
       </c>
       <c r="C532" t="inlineStr">
         <is>
-          <t>25351234613202211</t>
+          <t>25351492777202253</t>
         </is>
       </c>
       <c r="D532" t="inlineStr">
@@ -14776,24 +14776,24 @@
       </c>
       <c r="E532" t="inlineStr">
         <is>
-          <t>22/08/2023</t>
+          <t>23/08/2023</t>
         </is>
       </c>
     </row>
     <row r="533">
       <c r="A533" t="inlineStr">
         <is>
-          <t>Centrient Pharmaceuticals Spain, S.A.</t>
+          <t>Ipca Laboratories Ltd.</t>
         </is>
       </c>
       <c r="B533" t="inlineStr">
         <is>
-          <t>cefalexina monoidratada</t>
+          <t>hidroclorotiazida</t>
         </is>
       </c>
       <c r="C533" t="inlineStr">
         <is>
-          <t>25351196266202122</t>
+          <t>25351234613202211</t>
         </is>
       </c>
       <c r="D533" t="inlineStr">
@@ -14803,88 +14803,88 @@
       </c>
       <c r="E533" t="inlineStr">
         <is>
-          <t>17/08/2023</t>
+          <t>22/08/2023</t>
         </is>
       </c>
     </row>
     <row r="534">
       <c r="A534" t="inlineStr">
         <is>
-          <t>Matrix Pharmacorp Private Limited</t>
+          <t>Centrient Pharmaceuticals Spain, S.A.</t>
         </is>
       </c>
       <c r="B534" t="inlineStr">
         <is>
-          <t>aciclovir</t>
+          <t>cefalexina monoidratada</t>
         </is>
       </c>
       <c r="C534" t="inlineStr">
         <is>
-          <t>25351247888202126</t>
+          <t>25351196266202122</t>
         </is>
       </c>
       <c r="D534" t="inlineStr">
         <is>
-          <t>004</t>
+          <t>001</t>
         </is>
       </c>
       <c r="E534" t="inlineStr">
         <is>
-          <t>04/08/2023</t>
+          <t>17/08/2023</t>
         </is>
       </c>
     </row>
     <row r="535">
       <c r="A535" t="inlineStr">
         <is>
-          <t>Solara Active Pharma Sciences Limited</t>
+          <t>Matrix Pharmacorp Private Limited</t>
         </is>
       </c>
       <c r="B535" t="inlineStr">
         <is>
-          <t>ibuprofeno</t>
+          <t>aciclovir</t>
         </is>
       </c>
       <c r="C535" t="inlineStr">
         <is>
-          <t>25351072240202351</t>
+          <t>25351247888202126</t>
         </is>
       </c>
       <c r="D535" t="inlineStr">
         <is>
-          <t>001.1</t>
+          <t>004</t>
         </is>
       </c>
       <c r="E535" t="inlineStr">
         <is>
-          <t>14/07/2023</t>
+          <t>04/08/2023</t>
         </is>
       </c>
     </row>
     <row r="536">
       <c r="A536" t="inlineStr">
         <is>
-          <t>Harman Finochem Limited</t>
+          <t>Solara Active Pharma Sciences Limited</t>
         </is>
       </c>
       <c r="B536" t="inlineStr">
         <is>
-          <t>cloridrato de metformina</t>
+          <t>ibuprofeno</t>
         </is>
       </c>
       <c r="C536" t="inlineStr">
         <is>
-          <t>25351583229202231</t>
+          <t>25351072240202351</t>
         </is>
       </c>
       <c r="D536" t="inlineStr">
         <is>
-          <t>001</t>
+          <t>001.1</t>
         </is>
       </c>
       <c r="E536" t="inlineStr">
         <is>
-          <t>11/07/2023</t>
+          <t>14/07/2023</t>
         </is>
       </c>
     </row>
@@ -14901,7 +14901,7 @@
       </c>
       <c r="C537" t="inlineStr">
         <is>
-          <t>25351165919202211</t>
+          <t>25351583229202231</t>
         </is>
       </c>
       <c r="D537" t="inlineStr">
@@ -14911,29 +14911,29 @@
       </c>
       <c r="E537" t="inlineStr">
         <is>
-          <t>06/07/2023</t>
+          <t>11/07/2023</t>
         </is>
       </c>
     </row>
     <row r="538">
       <c r="A538" t="inlineStr">
         <is>
-          <t>Msn Organics Private Limited</t>
+          <t>Harman Finochem Limited</t>
         </is>
       </c>
       <c r="B538" t="inlineStr">
         <is>
-          <t>parecoxibe sódico</t>
+          <t>cloridrato de metformina</t>
         </is>
       </c>
       <c r="C538" t="inlineStr">
         <is>
-          <t>25351000511202296</t>
+          <t>25351165919202211</t>
         </is>
       </c>
       <c r="D538" t="inlineStr">
         <is>
-          <t>002</t>
+          <t>001</t>
         </is>
       </c>
       <c r="E538" t="inlineStr">
@@ -14945,17 +14945,17 @@
     <row r="539">
       <c r="A539" t="inlineStr">
         <is>
-          <t>Msn Pharmachem Private Limited</t>
+          <t>Msn Organics Private Limited</t>
         </is>
       </c>
       <c r="B539" t="inlineStr">
         <is>
-          <t>fosfato de sitagliptina monoidratado</t>
+          <t>parecoxibe sódico</t>
         </is>
       </c>
       <c r="C539" t="inlineStr">
         <is>
-          <t>25351745532202153</t>
+          <t>25351000511202296</t>
         </is>
       </c>
       <c r="D539" t="inlineStr">
@@ -14965,267 +14965,267 @@
       </c>
       <c r="E539" t="inlineStr">
         <is>
-          <t>23/06/2023</t>
+          <t>06/07/2023</t>
         </is>
       </c>
     </row>
     <row r="540">
       <c r="A540" t="inlineStr">
         <is>
-          <t>Alivus Life Sciences Limited</t>
+          <t>Msn Pharmachem Private Limited</t>
         </is>
       </c>
       <c r="B540" t="inlineStr">
         <is>
-          <t>hemitartarato de zolpidem</t>
+          <t>fosfato de sitagliptina monoidratado</t>
         </is>
       </c>
       <c r="C540" t="inlineStr">
         <is>
-          <t>25351851362202145</t>
+          <t>25351745532202153</t>
         </is>
       </c>
       <c r="D540" t="inlineStr">
         <is>
-          <t>003</t>
+          <t>002</t>
         </is>
       </c>
       <c r="E540" t="inlineStr">
         <is>
-          <t>20/06/2023</t>
+          <t>23/06/2023</t>
         </is>
       </c>
     </row>
     <row r="541">
       <c r="A541" t="inlineStr">
         <is>
-          <t>Macfarlan Smith Limited</t>
+          <t>Alivus Life Sciences Limited</t>
         </is>
       </c>
       <c r="B541" t="inlineStr">
         <is>
-          <t>fosfato de codeína hemi-hidratado</t>
+          <t>hemitartarato de zolpidem</t>
         </is>
       </c>
       <c r="C541" t="inlineStr">
         <is>
-          <t>25351214747202127</t>
+          <t>25351851362202145</t>
         </is>
       </c>
       <c r="D541" t="inlineStr">
         <is>
-          <t>001</t>
+          <t>003</t>
         </is>
       </c>
       <c r="E541" t="inlineStr">
         <is>
-          <t>30/05/2023</t>
+          <t>20/06/2023</t>
         </is>
       </c>
     </row>
     <row r="542">
       <c r="A542" t="inlineStr">
         <is>
-          <t>Aspen Oss B.V.</t>
+          <t>Macfarlan Smith Limited</t>
         </is>
       </c>
       <c r="B542" t="inlineStr">
         <is>
-          <t>ocitocina</t>
+          <t>fosfato de codeína hemi-hidratado</t>
         </is>
       </c>
       <c r="C542" t="inlineStr">
         <is>
-          <t>25351762016202193</t>
+          <t>25351214747202127</t>
         </is>
       </c>
       <c r="D542" t="inlineStr">
         <is>
-          <t>002</t>
+          <t>001</t>
         </is>
       </c>
       <c r="E542" t="inlineStr">
         <is>
-          <t>29/05/2023</t>
+          <t>30/05/2023</t>
         </is>
       </c>
     </row>
     <row r="543">
       <c r="A543" t="inlineStr">
         <is>
-          <t>Sinopharm Weiqida Pharmaceutical Co., Ltd.</t>
+          <t>Aspen Oss B.V.</t>
         </is>
       </c>
       <c r="B543" t="inlineStr">
         <is>
-          <t>ceftriaxona dissódica hemieptaidratada</t>
+          <t>ocitocina</t>
         </is>
       </c>
       <c r="C543" t="inlineStr">
         <is>
-          <t>25351464371202108</t>
+          <t>25351762016202193</t>
         </is>
       </c>
       <c r="D543" t="inlineStr">
         <is>
-          <t>001</t>
+          <t>002</t>
         </is>
       </c>
       <c r="E543" t="inlineStr">
         <is>
-          <t>26/05/2023</t>
+          <t>29/05/2023</t>
         </is>
       </c>
     </row>
     <row r="544">
       <c r="A544" t="inlineStr">
         <is>
-          <t>Chemo Do Brasil Comércio De Farmoquímicos Ltda</t>
+          <t>Sinopharm Weiqida Pharmaceutical Co., Ltd.</t>
         </is>
       </c>
       <c r="B544" t="inlineStr">
         <is>
-          <t>drospirenona</t>
+          <t>ceftriaxona dissódica hemieptaidratada</t>
         </is>
       </c>
       <c r="C544" t="inlineStr">
         <is>
-          <t>25351273206202211</t>
+          <t>25351464371202108</t>
         </is>
       </c>
       <c r="D544" t="inlineStr">
         <is>
-          <t>005</t>
+          <t>001</t>
         </is>
       </c>
       <c r="E544" t="inlineStr">
         <is>
-          <t>23/05/2023</t>
+          <t>26/05/2023</t>
         </is>
       </c>
     </row>
     <row r="545">
       <c r="A545" t="inlineStr">
         <is>
-          <t>Shandong Anshun Pharmaceutical Co., Ltd.</t>
+          <t>Chemo Do Brasil Comércio De Farmoquímicos Ltda</t>
         </is>
       </c>
       <c r="B545" t="inlineStr">
         <is>
-          <t>tazobactam</t>
+          <t>drospirenona</t>
         </is>
       </c>
       <c r="C545" t="inlineStr">
         <is>
-          <t>25351088152202291</t>
+          <t>25351273206202211</t>
         </is>
       </c>
       <c r="D545" t="inlineStr">
         <is>
-          <t>001.1</t>
+          <t>005</t>
         </is>
       </c>
       <c r="E545" t="inlineStr">
         <is>
-          <t>09/05/2023</t>
+          <t>23/05/2023</t>
         </is>
       </c>
     </row>
     <row r="546">
       <c r="A546" t="inlineStr">
         <is>
-          <t>Qilu Antibiotics Pharmaceutical Co., Ltd.</t>
+          <t>Shandong Anshun Pharmaceutical Co., Ltd.</t>
         </is>
       </c>
       <c r="B546" t="inlineStr">
         <is>
-          <t>ceftriaxona dissódica hemieptaidratada</t>
+          <t>tazobactam</t>
         </is>
       </c>
       <c r="C546" t="inlineStr">
         <is>
-          <t>25351535972202102</t>
+          <t>25351088152202291</t>
         </is>
       </c>
       <c r="D546" t="inlineStr">
         <is>
-          <t>002.1</t>
+          <t>001.1</t>
         </is>
       </c>
       <c r="E546" t="inlineStr">
         <is>
-          <t>08/05/2023</t>
+          <t>09/05/2023</t>
         </is>
       </c>
     </row>
     <row r="547">
       <c r="A547" t="inlineStr">
         <is>
-          <t>Antibióticos Do Brasil Ltda</t>
+          <t>Qilu Antibiotics Pharmaceutical Co., Ltd.</t>
         </is>
       </c>
       <c r="B547" t="inlineStr">
         <is>
-          <t>ceftazidima pentaidratada</t>
+          <t>ceftriaxona dissódica hemieptaidratada</t>
         </is>
       </c>
       <c r="C547" t="inlineStr">
         <is>
-          <t>25351063708202155</t>
+          <t>25351535972202102</t>
         </is>
       </c>
       <c r="D547" t="inlineStr">
         <is>
-          <t>001</t>
+          <t>002.1</t>
         </is>
       </c>
       <c r="E547" t="inlineStr">
         <is>
-          <t>02/05/2023</t>
+          <t>08/05/2023</t>
         </is>
       </c>
     </row>
     <row r="548">
       <c r="A548" t="inlineStr">
         <is>
-          <t>Farmson Basic Drugs Private Limited</t>
+          <t>Antibióticos Do Brasil Ltda</t>
         </is>
       </c>
       <c r="B548" t="inlineStr">
         <is>
-          <t>paracetamol</t>
+          <t>ceftazidima pentaidratada</t>
         </is>
       </c>
       <c r="C548" t="inlineStr">
         <is>
-          <t>25351898107202166</t>
+          <t>25351063708202155</t>
         </is>
       </c>
       <c r="D548" t="inlineStr">
         <is>
-          <t>002</t>
+          <t>001</t>
         </is>
       </c>
       <c r="E548" t="inlineStr">
         <is>
-          <t>27/04/2023</t>
+          <t>02/05/2023</t>
         </is>
       </c>
     </row>
     <row r="549">
       <c r="A549" t="inlineStr">
         <is>
-          <t>Alivus Life Sciences Limited</t>
+          <t>Farmson Basic Drugs Private Limited</t>
         </is>
       </c>
       <c r="B549" t="inlineStr">
         <is>
-          <t>etoricoxibe</t>
+          <t>paracetamol</t>
         </is>
       </c>
       <c r="C549" t="inlineStr">
         <is>
-          <t>25351514251202151</t>
+          <t>25351898107202166</t>
         </is>
       </c>
       <c r="D549" t="inlineStr">
@@ -15235,51 +15235,51 @@
       </c>
       <c r="E549" t="inlineStr">
         <is>
-          <t>26/04/2023</t>
+          <t>27/04/2023</t>
         </is>
       </c>
     </row>
     <row r="550">
       <c r="A550" t="inlineStr">
         <is>
-          <t>Gland Pharma Limited</t>
+          <t>Alivus Life Sciences Limited</t>
         </is>
       </c>
       <c r="B550" t="inlineStr">
         <is>
-          <t>brometo de rocurônio</t>
+          <t>etoricoxibe</t>
         </is>
       </c>
       <c r="C550" t="inlineStr">
         <is>
-          <t>25351037183202283</t>
+          <t>25351514251202151</t>
         </is>
       </c>
       <c r="D550" t="inlineStr">
         <is>
-          <t>001</t>
+          <t>002</t>
         </is>
       </c>
       <c r="E550" t="inlineStr">
         <is>
-          <t>18/04/2023</t>
+          <t>26/04/2023</t>
         </is>
       </c>
     </row>
     <row r="551">
       <c r="A551" t="inlineStr">
         <is>
-          <t>Intas Pharmaceuticals Limited</t>
+          <t>Gland Pharma Limited</t>
         </is>
       </c>
       <c r="B551" t="inlineStr">
         <is>
-          <t>cloridrato de doxorrubicina</t>
+          <t>brometo de rocurônio</t>
         </is>
       </c>
       <c r="C551" t="inlineStr">
         <is>
-          <t>25351604159202181</t>
+          <t>25351037183202283</t>
         </is>
       </c>
       <c r="D551" t="inlineStr">
@@ -15296,17 +15296,17 @@
     <row r="552">
       <c r="A552" t="inlineStr">
         <is>
-          <t>Janssen-Cilag Farmaceutica Ltda</t>
+          <t>Intas Pharmaceuticals Limited</t>
         </is>
       </c>
       <c r="B552" t="inlineStr">
         <is>
-          <t>cloridrato de rilpivirina</t>
+          <t>cloridrato de doxorrubicina</t>
         </is>
       </c>
       <c r="C552" t="inlineStr">
         <is>
-          <t>25351221052202100</t>
+          <t>25351604159202181</t>
         </is>
       </c>
       <c r="D552" t="inlineStr">
@@ -15316,7 +15316,7 @@
       </c>
       <c r="E552" t="inlineStr">
         <is>
-          <t>14/04/2023</t>
+          <t>18/04/2023</t>
         </is>
       </c>
     </row>
@@ -15328,44 +15328,44 @@
       </c>
       <c r="B553" t="inlineStr">
         <is>
-          <t>rilpivirina</t>
+          <t>cloridrato de rilpivirina</t>
         </is>
       </c>
       <c r="C553" t="inlineStr">
         <is>
-          <t>25351381305202195</t>
+          <t>25351221052202100</t>
         </is>
       </c>
       <c r="D553" t="inlineStr">
         <is>
-          <t>002</t>
+          <t>001</t>
         </is>
       </c>
       <c r="E553" t="inlineStr">
         <is>
-          <t>05/04/2023</t>
+          <t>14/04/2023</t>
         </is>
       </c>
     </row>
     <row r="554">
       <c r="A554" t="inlineStr">
         <is>
-          <t>Alembic Pharmaceuticals Limited</t>
+          <t>Janssen-Cilag Farmaceutica Ltda</t>
         </is>
       </c>
       <c r="B554" t="inlineStr">
         <is>
-          <t>etoricoxibe</t>
+          <t>rilpivirina</t>
         </is>
       </c>
       <c r="C554" t="inlineStr">
         <is>
-          <t>25351459577202116</t>
+          <t>25351381305202195</t>
         </is>
       </c>
       <c r="D554" t="inlineStr">
         <is>
-          <t>001</t>
+          <t>002</t>
         </is>
       </c>
       <c r="E554" t="inlineStr">
@@ -15377,71 +15377,71 @@
     <row r="555">
       <c r="A555" t="inlineStr">
         <is>
-          <t>Shandong Anshun Pharmaceutical Co., Ltd.</t>
+          <t>Alembic Pharmaceuticals Limited</t>
         </is>
       </c>
       <c r="B555" t="inlineStr">
         <is>
-          <t>piperacilina monoidratada</t>
+          <t>etoricoxibe</t>
         </is>
       </c>
       <c r="C555" t="inlineStr">
         <is>
-          <t>25351088151202246</t>
+          <t>25351459577202116</t>
         </is>
       </c>
       <c r="D555" t="inlineStr">
         <is>
-          <t>001.1</t>
+          <t>001</t>
         </is>
       </c>
       <c r="E555" t="inlineStr">
         <is>
-          <t>30/03/2023</t>
+          <t>05/04/2023</t>
         </is>
       </c>
     </row>
     <row r="556">
       <c r="A556" t="inlineStr">
         <is>
-          <t>Chemo Do Brasil Comércio De Farmoquímicos Ltda</t>
+          <t>Shandong Anshun Pharmaceutical Co., Ltd.</t>
         </is>
       </c>
       <c r="B556" t="inlineStr">
         <is>
-          <t>etinilestradiol</t>
+          <t>piperacilina monoidratada</t>
         </is>
       </c>
       <c r="C556" t="inlineStr">
         <is>
-          <t>25351788882202295</t>
+          <t>25351088151202246</t>
         </is>
       </c>
       <c r="D556" t="inlineStr">
         <is>
-          <t>002</t>
+          <t>001.1</t>
         </is>
       </c>
       <c r="E556" t="inlineStr">
         <is>
-          <t>23/03/2023</t>
+          <t>30/03/2023</t>
         </is>
       </c>
     </row>
     <row r="557">
       <c r="A557" t="inlineStr">
         <is>
-          <t>Zhejiang Guobang Pharmaceutical Co., Ltd</t>
+          <t>Chemo Do Brasil Comércio De Farmoquímicos Ltda</t>
         </is>
       </c>
       <c r="B557" t="inlineStr">
         <is>
-          <t>azitromicina di-hidratada</t>
+          <t>etinilestradiol</t>
         </is>
       </c>
       <c r="C557" t="inlineStr">
         <is>
-          <t>25351198490202159</t>
+          <t>25351788882202295</t>
         </is>
       </c>
       <c r="D557" t="inlineStr">
@@ -15451,29 +15451,29 @@
       </c>
       <c r="E557" t="inlineStr">
         <is>
-          <t>23/02/2023</t>
+          <t>23/03/2023</t>
         </is>
       </c>
     </row>
     <row r="558">
       <c r="A558" t="inlineStr">
         <is>
-          <t>Intas Pharmaceuticals Limited</t>
+          <t>Zhejiang Guobang Pharmaceutical Co., Ltd</t>
         </is>
       </c>
       <c r="B558" t="inlineStr">
         <is>
-          <t>fampridina</t>
+          <t>azitromicina di-hidratada</t>
         </is>
       </c>
       <c r="C558" t="inlineStr">
         <is>
-          <t>25351007864202217</t>
+          <t>25351198490202159</t>
         </is>
       </c>
       <c r="D558" t="inlineStr">
         <is>
-          <t>001</t>
+          <t>002</t>
         </is>
       </c>
       <c r="E558" t="inlineStr">
@@ -15485,17 +15485,17 @@
     <row r="559">
       <c r="A559" t="inlineStr">
         <is>
-          <t>Hetero Labs Limited</t>
+          <t>Intas Pharmaceuticals Limited</t>
         </is>
       </c>
       <c r="B559" t="inlineStr">
         <is>
-          <t>bicalutamida</t>
+          <t>fampridina</t>
         </is>
       </c>
       <c r="C559" t="inlineStr">
         <is>
-          <t>25351159727202003</t>
+          <t>25351007864202217</t>
         </is>
       </c>
       <c r="D559" t="inlineStr">
@@ -15505,24 +15505,24 @@
       </c>
       <c r="E559" t="inlineStr">
         <is>
-          <t>15/02/2023</t>
+          <t>23/02/2023</t>
         </is>
       </c>
     </row>
     <row r="560">
       <c r="A560" t="inlineStr">
         <is>
-          <t>Msn Laboratories Private Limited</t>
+          <t>Hetero Labs Limited</t>
         </is>
       </c>
       <c r="B560" t="inlineStr">
         <is>
-          <t>enzalutamida</t>
+          <t>bicalutamida</t>
         </is>
       </c>
       <c r="C560" t="inlineStr">
         <is>
-          <t>25351042982202191</t>
+          <t>25351159727202003</t>
         </is>
       </c>
       <c r="D560" t="inlineStr">
@@ -15532,24 +15532,24 @@
       </c>
       <c r="E560" t="inlineStr">
         <is>
-          <t>13/02/2023</t>
+          <t>15/02/2023</t>
         </is>
       </c>
     </row>
     <row r="561">
       <c r="A561" t="inlineStr">
         <is>
-          <t>Fersinsa Gb S.A. De C.V.</t>
+          <t>Msn Laboratories Private Limited</t>
         </is>
       </c>
       <c r="B561" t="inlineStr">
         <is>
-          <t>benzilpenicilina potássica</t>
+          <t>enzalutamida</t>
         </is>
       </c>
       <c r="C561" t="inlineStr">
         <is>
-          <t>25351881526202169</t>
+          <t>25351042982202191</t>
         </is>
       </c>
       <c r="D561" t="inlineStr">
@@ -15559,24 +15559,24 @@
       </c>
       <c r="E561" t="inlineStr">
         <is>
-          <t>01/02/2023</t>
+          <t>13/02/2023</t>
         </is>
       </c>
     </row>
     <row r="562">
       <c r="A562" t="inlineStr">
         <is>
-          <t>Transo-Pharm Handels-Gmbh</t>
+          <t>Fersinsa Gb S.A. De C.V.</t>
         </is>
       </c>
       <c r="B562" t="inlineStr">
         <is>
-          <t>cloridrato de doxorrubicina</t>
+          <t>benzilpenicilina potássica</t>
         </is>
       </c>
       <c r="C562" t="inlineStr">
         <is>
-          <t>25351666895202123</t>
+          <t>25351881526202169</t>
         </is>
       </c>
       <c r="D562" t="inlineStr">
@@ -15593,17 +15593,17 @@
     <row r="563">
       <c r="A563" t="inlineStr">
         <is>
-          <t>Cyg Biotech Qumica &amp; Farmaceutica Ltda.</t>
+          <t>Transo-Pharm Handels-Gmbh</t>
         </is>
       </c>
       <c r="B563" t="inlineStr">
         <is>
-          <t>carbonato de lítio</t>
+          <t>cloridrato de doxorrubicina</t>
         </is>
       </c>
       <c r="C563" t="inlineStr">
         <is>
-          <t>25351759475202190</t>
+          <t>25351666895202123</t>
         </is>
       </c>
       <c r="D563" t="inlineStr">
@@ -15613,56 +15613,56 @@
       </c>
       <c r="E563" t="inlineStr">
         <is>
-          <t>28/12/2022</t>
+          <t>01/02/2023</t>
         </is>
       </c>
     </row>
     <row r="564">
       <c r="A564" t="inlineStr">
         <is>
-          <t>Zhejiang Hisun Pharmaceutical Co., Ltd.</t>
+          <t>Cyg Biotech Qumica &amp; Farmaceutica Ltda.</t>
         </is>
       </c>
       <c r="B564" t="inlineStr">
         <is>
-          <t>tigeciclina</t>
+          <t>carbonato de lítio</t>
         </is>
       </c>
       <c r="C564" t="inlineStr">
         <is>
-          <t>25351970820202063</t>
+          <t>25351759475202190</t>
         </is>
       </c>
       <c r="D564" t="inlineStr">
         <is>
-          <t>002</t>
+          <t>001</t>
         </is>
       </c>
       <c r="E564" t="inlineStr">
         <is>
-          <t>07/12/2022</t>
+          <t>28/12/2022</t>
         </is>
       </c>
     </row>
     <row r="565">
       <c r="A565" t="inlineStr">
         <is>
-          <t>Alembic Pharmaceuticals Limited</t>
+          <t>Zhejiang Hisun Pharmaceutical Co., Ltd.</t>
         </is>
       </c>
       <c r="B565" t="inlineStr">
         <is>
-          <t>succinato de desvenlafaxina monoidratado</t>
+          <t>tigeciclina</t>
         </is>
       </c>
       <c r="C565" t="inlineStr">
         <is>
-          <t>25351114763202111</t>
+          <t>25351970820202063</t>
         </is>
       </c>
       <c r="D565" t="inlineStr">
         <is>
-          <t>001.1</t>
+          <t>002</t>
         </is>
       </c>
       <c r="E565" t="inlineStr">
@@ -15674,27 +15674,27 @@
     <row r="566">
       <c r="A566" t="inlineStr">
         <is>
-          <t>Msn Laboratories Private Limited</t>
+          <t>Alembic Pharmaceuticals Limited</t>
         </is>
       </c>
       <c r="B566" t="inlineStr">
         <is>
-          <t>gefitinibe</t>
+          <t>succinato de desvenlafaxina monoidratado</t>
         </is>
       </c>
       <c r="C566" t="inlineStr">
         <is>
-          <t>25351199392202139</t>
+          <t>25351114763202111</t>
         </is>
       </c>
       <c r="D566" t="inlineStr">
         <is>
-          <t>001</t>
+          <t>001.1</t>
         </is>
       </c>
       <c r="E566" t="inlineStr">
         <is>
-          <t>16/11/2022</t>
+          <t>07/12/2022</t>
         </is>
       </c>
     </row>
@@ -15706,12 +15706,12 @@
       </c>
       <c r="B567" t="inlineStr">
         <is>
-          <t>esilato de nintedanibe</t>
+          <t>gefitinibe</t>
         </is>
       </c>
       <c r="C567" t="inlineStr">
         <is>
-          <t>25351382611202068</t>
+          <t>25351199392202139</t>
         </is>
       </c>
       <c r="D567" t="inlineStr">
@@ -15721,132 +15721,132 @@
       </c>
       <c r="E567" t="inlineStr">
         <is>
-          <t>10/11/2022</t>
+          <t>16/11/2022</t>
         </is>
       </c>
     </row>
     <row r="568">
       <c r="A568" t="inlineStr">
         <is>
-          <t>Harman Finochem Limited</t>
+          <t>Msn Laboratories Private Limited</t>
         </is>
       </c>
       <c r="B568" t="inlineStr">
         <is>
-          <t>cloridrato de metformina</t>
+          <t>esilato de nintedanibe</t>
         </is>
       </c>
       <c r="C568" t="inlineStr">
         <is>
-          <t>25351223837202117</t>
+          <t>25351382611202068</t>
         </is>
       </c>
       <c r="D568" t="inlineStr">
         <is>
-          <t>003</t>
+          <t>001</t>
         </is>
       </c>
       <c r="E568" t="inlineStr">
         <is>
-          <t>25/10/2022</t>
+          <t>10/11/2022</t>
         </is>
       </c>
     </row>
     <row r="569">
       <c r="A569" t="inlineStr">
         <is>
-          <t>Biocon Limited</t>
+          <t>Harman Finochem Limited</t>
         </is>
       </c>
       <c r="B569" t="inlineStr">
         <is>
-          <t>everolimo</t>
+          <t>cloridrato de metformina</t>
         </is>
       </c>
       <c r="C569" t="inlineStr">
         <is>
-          <t>25351692063202162</t>
+          <t>25351223837202117</t>
         </is>
       </c>
       <c r="D569" t="inlineStr">
         <is>
-          <t>002</t>
+          <t>003</t>
         </is>
       </c>
       <c r="E569" t="inlineStr">
         <is>
-          <t>21/10/2022</t>
+          <t>25/10/2022</t>
         </is>
       </c>
     </row>
     <row r="570">
       <c r="A570" t="inlineStr">
         <is>
-          <t>Synthimed Labs Private Limited</t>
+          <t>Biocon Limited</t>
         </is>
       </c>
       <c r="B570" t="inlineStr">
         <is>
-          <t>claritromicina</t>
+          <t>everolimo</t>
         </is>
       </c>
       <c r="C570" t="inlineStr">
         <is>
-          <t>25351517246202281</t>
+          <t>25351692063202162</t>
         </is>
       </c>
       <c r="D570" t="inlineStr">
         <is>
-          <t>003</t>
+          <t>002</t>
         </is>
       </c>
       <c r="E570" t="inlineStr">
         <is>
-          <t>18/10/2022</t>
+          <t>21/10/2022</t>
         </is>
       </c>
     </row>
     <row r="571">
       <c r="A571" t="inlineStr">
         <is>
-          <t>Shilpa Pharma Lifesciences Limited</t>
+          <t>Synthimed Labs Private Limited</t>
         </is>
       </c>
       <c r="B571" t="inlineStr">
         <is>
-          <t>cloridrato de bendamustina monoidratada</t>
+          <t>claritromicina</t>
         </is>
       </c>
       <c r="C571" t="inlineStr">
         <is>
-          <t>25351748374202193</t>
+          <t>25351517246202281</t>
         </is>
       </c>
       <c r="D571" t="inlineStr">
         <is>
-          <t>001</t>
+          <t>003</t>
         </is>
       </c>
       <c r="E571" t="inlineStr">
         <is>
-          <t>14/10/2022</t>
+          <t>18/10/2022</t>
         </is>
       </c>
     </row>
     <row r="572">
       <c r="A572" t="inlineStr">
         <is>
-          <t>Msn Laboratories Private Limited</t>
+          <t>Shilpa Pharma Lifesciences Limited</t>
         </is>
       </c>
       <c r="B572" t="inlineStr">
         <is>
-          <t>tosilato de sorafenibe</t>
+          <t>cloridrato de bendamustina monoidratada</t>
         </is>
       </c>
       <c r="C572" t="inlineStr">
         <is>
-          <t>25351915465202141</t>
+          <t>25351748374202193</t>
         </is>
       </c>
       <c r="D572" t="inlineStr">
@@ -15856,24 +15856,24 @@
       </c>
       <c r="E572" t="inlineStr">
         <is>
-          <t>11/10/2022</t>
+          <t>14/10/2022</t>
         </is>
       </c>
     </row>
     <row r="573">
       <c r="A573" t="inlineStr">
         <is>
-          <t>Sun Pharmaceutical Industries Limited</t>
+          <t>Msn Laboratories Private Limited</t>
         </is>
       </c>
       <c r="B573" t="inlineStr">
         <is>
-          <t>vildagliptina</t>
+          <t>tosilato de sorafenibe</t>
         </is>
       </c>
       <c r="C573" t="inlineStr">
         <is>
-          <t>25351063743202255</t>
+          <t>25351915465202141</t>
         </is>
       </c>
       <c r="D573" t="inlineStr">
@@ -15883,132 +15883,132 @@
       </c>
       <c r="E573" t="inlineStr">
         <is>
-          <t>10/10/2022</t>
+          <t>11/10/2022</t>
         </is>
       </c>
     </row>
     <row r="574">
       <c r="A574" t="inlineStr">
         <is>
-          <t>Zhejiang Charioteer Pharmaceutical Co., Ltd.</t>
+          <t>Sun Pharmaceutical Industries Limited</t>
         </is>
       </c>
       <c r="B574" t="inlineStr">
         <is>
-          <t>aciclovir</t>
+          <t>vildagliptina</t>
         </is>
       </c>
       <c r="C574" t="inlineStr">
         <is>
-          <t>25351308050202116</t>
+          <t>25351063743202255</t>
         </is>
       </c>
       <c r="D574" t="inlineStr">
         <is>
-          <t>002.1</t>
+          <t>001</t>
         </is>
       </c>
       <c r="E574" t="inlineStr">
         <is>
-          <t>12/09/2022</t>
+          <t>10/10/2022</t>
         </is>
       </c>
     </row>
     <row r="575">
       <c r="A575" t="inlineStr">
         <is>
-          <t>Shilpa Pharma Lifesciences Limited</t>
+          <t>Zhejiang Charioteer Pharmaceutical Co., Ltd.</t>
         </is>
       </c>
       <c r="B575" t="inlineStr">
         <is>
-          <t>bussulfano</t>
+          <t>aciclovir</t>
         </is>
       </c>
       <c r="C575" t="inlineStr">
         <is>
-          <t>25351653813202181</t>
+          <t>25351308050202116</t>
         </is>
       </c>
       <c r="D575" t="inlineStr">
         <is>
-          <t>002</t>
+          <t>002.1</t>
         </is>
       </c>
       <c r="E575" t="inlineStr">
         <is>
-          <t>20/08/2022</t>
+          <t>12/09/2022</t>
         </is>
       </c>
     </row>
     <row r="576">
       <c r="A576" t="inlineStr">
         <is>
-          <t>Honour Lab Limited</t>
+          <t>Shilpa Pharma Lifesciences Limited</t>
         </is>
       </c>
       <c r="B576" t="inlineStr">
         <is>
-          <t>fosfato de sitagliptina</t>
+          <t>bussulfano</t>
         </is>
       </c>
       <c r="C576" t="inlineStr">
         <is>
-          <t>25351333869202031</t>
+          <t>25351653813202181</t>
         </is>
       </c>
       <c r="D576" t="inlineStr">
         <is>
-          <t>001</t>
+          <t>002</t>
         </is>
       </c>
       <c r="E576" t="inlineStr">
         <is>
-          <t>16/08/2022</t>
+          <t>20/08/2022</t>
         </is>
       </c>
     </row>
     <row r="577">
       <c r="A577" t="inlineStr">
         <is>
-          <t>Fersinsa Gb S.A. De C.V.</t>
+          <t>Honour Lab Limited</t>
         </is>
       </c>
       <c r="B577" t="inlineStr">
         <is>
-          <t>amoxicilina tri-hidratada</t>
+          <t>fosfato de sitagliptina</t>
         </is>
       </c>
       <c r="C577" t="inlineStr">
         <is>
-          <t>25351533263202001</t>
+          <t>25351333869202031</t>
         </is>
       </c>
       <c r="D577" t="inlineStr">
         <is>
-          <t>002</t>
+          <t>001</t>
         </is>
       </c>
       <c r="E577" t="inlineStr">
         <is>
-          <t>08/08/2022</t>
+          <t>16/08/2022</t>
         </is>
       </c>
     </row>
     <row r="578">
       <c r="A578" t="inlineStr">
         <is>
-          <t>Tapi Brazil Ltda</t>
+          <t>Fersinsa Gb S.A. De C.V.</t>
         </is>
       </c>
       <c r="B578" t="inlineStr">
         <is>
-          <t>cloridrato de memantina</t>
+          <t>amoxicilina tri-hidratada</t>
         </is>
       </c>
       <c r="C578" t="inlineStr">
         <is>
-          <t>25351537007202166</t>
+          <t>25351533263202001</t>
         </is>
       </c>
       <c r="D578" t="inlineStr">
@@ -16018,51 +16018,51 @@
       </c>
       <c r="E578" t="inlineStr">
         <is>
-          <t>18/07/2022</t>
+          <t>08/08/2022</t>
         </is>
       </c>
     </row>
     <row r="579">
       <c r="A579" t="inlineStr">
         <is>
-          <t>Alembic Pharmaceuticals Limited</t>
+          <t>Tapi Brazil Ltda</t>
         </is>
       </c>
       <c r="B579" t="inlineStr">
         <is>
-          <t>vildagliptina</t>
+          <t>cloridrato de memantina</t>
         </is>
       </c>
       <c r="C579" t="inlineStr">
         <is>
-          <t>25351871278202067</t>
+          <t>25351537007202166</t>
         </is>
       </c>
       <c r="D579" t="inlineStr">
         <is>
-          <t>001</t>
+          <t>002</t>
         </is>
       </c>
       <c r="E579" t="inlineStr">
         <is>
-          <t>04/04/2022</t>
+          <t>18/07/2022</t>
         </is>
       </c>
     </row>
     <row r="580">
       <c r="A580" t="inlineStr">
         <is>
-          <t>Msn Laboratories Private Limited</t>
+          <t>Alembic Pharmaceuticals Limited</t>
         </is>
       </c>
       <c r="B580" t="inlineStr">
         <is>
-          <t>rosuvastatina cálcica</t>
+          <t>vildagliptina</t>
         </is>
       </c>
       <c r="C580" t="inlineStr">
         <is>
-          <t>25351322289202018</t>
+          <t>25351871278202067</t>
         </is>
       </c>
       <c r="D580" t="inlineStr">
@@ -16072,32 +16072,59 @@
       </c>
       <c r="E580" t="inlineStr">
         <is>
-          <t>16/03/2022</t>
+          <t>04/04/2022</t>
         </is>
       </c>
     </row>
     <row r="581">
       <c r="A581" t="inlineStr">
         <is>
+          <t>Msn Laboratories Private Limited</t>
+        </is>
+      </c>
+      <c r="B581" t="inlineStr">
+        <is>
+          <t>rosuvastatina cálcica</t>
+        </is>
+      </c>
+      <c r="C581" t="inlineStr">
+        <is>
+          <t>25351322289202018</t>
+        </is>
+      </c>
+      <c r="D581" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="E581" t="inlineStr">
+        <is>
+          <t>16/03/2022</t>
+        </is>
+      </c>
+    </row>
+    <row r="582">
+      <c r="A582" t="inlineStr">
+        <is>
           <t>Viyash Scientific Limited</t>
         </is>
       </c>
-      <c r="B581" t="inlineStr">
+      <c r="B582" t="inlineStr">
         <is>
           <t>cloridrato  de ondansetrona di-hidratado</t>
         </is>
       </c>
-      <c r="C581" t="inlineStr">
+      <c r="C582" t="inlineStr">
         <is>
           <t>25351163773202180</t>
         </is>
       </c>
-      <c r="D581" t="inlineStr">
+      <c r="D582" t="inlineStr">
         <is>
           <t>001.1</t>
         </is>
       </c>
-      <c r="E581" t="inlineStr">
+      <c r="E582" t="inlineStr">
         <is>
           <t>23/02/2022</t>
         </is>

</xml_diff>

<commit_message>
Atualiza lista de CADIFAs deferidas (execução automática)
Nenhuma linha nova desde a última execução (612 CADIFAs deferidas).
</commit_message>
<xml_diff>
--- a/cadifa_completo.xlsx
+++ b/cadifa_completo.xlsx
@@ -446,17 +446,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Bec Chemicals Private Limited</t>
+          <t>Dr Reddys Farmacêutica Do Brasil Ltda</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>cetoprofeno</t>
+          <t>gatifloxacino</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>25351184842202351</t>
+          <t>25351755793202343</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -466,24 +466,24 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>21/08/2026</t>
+          <t>25/08/2026</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Ami Lifesciences Private Limited</t>
+          <t>Kissei Pharmaceutical Co., Ltd.</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>tadalafila</t>
+          <t>linzagolixato de colina</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>25351299954202496</t>
+          <t>25351399700202477</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -493,24 +493,24 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>20/08/2026</t>
+          <t>25/08/2026</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Kissei Pharmaceutical Co., Ltd.</t>
+          <t>Ami Lifesciences Private Limited</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>linzagolixato de colina</t>
+          <t>tadalafila</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>25351399700202477</t>
+          <t>25351299954202496</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -520,24 +520,24 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>20/08/2026</t>
+          <t>25/08/2026</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Ipca Laboratories Ltd.</t>
+          <t>Heraeus Deutschland Gmbh &amp; Co. Kg</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>hidroclorotiazida</t>
+          <t>cloridrato do ácido aminolevulínico</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>25351227277202595</t>
+          <t>25351145024202502</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -547,24 +547,24 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>19/08/2026</t>
+          <t>25/08/2026</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Honour Lab Limited</t>
+          <t>Zydus Lifesciences Limited</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>brexpiprazol</t>
+          <t>bromidrato de vortioxetina</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>25351075968202505</t>
+          <t>25351141871202590</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -574,24 +574,24 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>19/08/2026</t>
+          <t>25/08/2026</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Heraeus Deutschland Gmbh &amp; Co. Kg</t>
+          <t>Bec Chemicals Private Limited</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>cloridrato do ácido aminolevulínico</t>
+          <t>cetoprofeno</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>25351145024202502</t>
+          <t>25351184842202351</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -601,24 +601,24 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>17/08/2026</t>
+          <t>25/08/2026</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Alivus Life Sciences Limited</t>
+          <t>Changzhou Pharmaceutical Factory</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>dicloridrato de levocetirizina</t>
+          <t>lenalidomida</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>25351372678202256</t>
+          <t>25351567349202372</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -628,7 +628,7 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>17/08/2026</t>
+          <t>25/08/2026</t>
         </is>
       </c>
     </row>
@@ -655,24 +655,24 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>17/08/2026</t>
+          <t>25/08/2026</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Changzhou Pharmaceutical Factory</t>
+          <t>Alivus Life Sciences Limited</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>lenalidomida</t>
+          <t>dicloridrato de levocetirizina</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>25351567349202372</t>
+          <t>25351372678202256</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -682,24 +682,24 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>17/08/2026</t>
+          <t>25/08/2026</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Ranke Química S.A.</t>
+          <t>Ipca Laboratories Ltd.</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>ebastina</t>
+          <t>hidroclorotiazida</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>25351570277202260</t>
+          <t>25351227277202595</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -709,24 +709,24 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>14/08/2026</t>
+          <t>25/08/2026</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Dr Reddys Farmacêutica Do Brasil Ltda</t>
+          <t>Ranke Química S.A.</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>levofloxacino hemi-hidratado</t>
+          <t>ebastina</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>25351957809202431</t>
+          <t>25351570277202260</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -736,24 +736,24 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>14/08/2026</t>
+          <t>25/08/2026</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Msn Laboratories Private Limited</t>
+          <t>Honour Lab Limited</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>carfilzomibe</t>
+          <t>ticagrelor</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>25351514099202297</t>
+          <t>25351156927202519</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -763,24 +763,24 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>14/08/2026</t>
+          <t>25/08/2026</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Shandong Anshun Pharmaceutical Co., Ltd.</t>
+          <t>Honour Lab Limited</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>piperacilina monoidratada</t>
+          <t>brexpiprazol</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>25351387641202494</t>
+          <t>25351075968202505</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -790,7 +790,7 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>14/08/2026</t>
+          <t>25/08/2026</t>
         </is>
       </c>
     </row>
@@ -802,12 +802,12 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>gatifloxacino</t>
+          <t>levofloxacino hemi-hidratado</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>25351755793202343</t>
+          <t>25351957809202431</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -824,17 +824,17 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Honour Lab Limited</t>
+          <t>Msn Laboratories Private Limited</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>ticagrelor</t>
+          <t>carfilzomibe</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>25351156927202519</t>
+          <t>25351514099202297</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -851,17 +851,17 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Alivus Life Sciences Limited</t>
+          <t>Shandong Anshun Pharmaceutical Co., Ltd.</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>cloridrato de lurasidona</t>
+          <t>piperacilina monoidratada</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>25351221146202413</t>
+          <t>25351387641202494</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -878,17 +878,17 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Malladi Drugs &amp; Pharmaceuticals Limited</t>
+          <t>Alivus Life Sciences Limited</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>cloridrato de pseudoefedrina</t>
+          <t>cloridrato de lurasidona</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>25351197304202326</t>
+          <t>25351221146202413</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -905,17 +905,17 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Zhuhai Rundu Pharmaceutical Co., Ltd.</t>
+          <t>Malladi Drugs &amp; Pharmaceuticals Limited</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>sacubitril valsartana sódica hidratada</t>
+          <t>cloridrato de pseudoefedrina</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>25351386758202451</t>
+          <t>25351197304202326</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -932,17 +932,17 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Zaklady Farmaceutyczne Polpharma S.A.</t>
+          <t>Zhuhai Rundu Pharmaceutical Co., Ltd.</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>ibandronato de sódio monoidratado</t>
+          <t>sacubitril valsartana sódica hidratada</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>25351154041202280</t>
+          <t>25351386758202451</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -959,17 +959,17 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Hubei Biocause Heilen Pharmaceutical Co., Ltd</t>
+          <t>Zaklady Farmaceutyczne Polpharma S.A.</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>dexibuprofeno</t>
+          <t>ibandronato de sódio monoidratado</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>25351138036202491</t>
+          <t>25351154041202280</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -986,17 +986,17 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Hetero Labs Limited</t>
+          <t>Hubei Biocause Heilen Pharmaceutical Co., Ltd</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>enzalutamida</t>
+          <t>dexibuprofeno</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>25351031614202541</t>
+          <t>25351138036202491</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -1013,17 +1013,17 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Zhejiang Huahai Pharmaceutical Co., Ltd.</t>
+          <t>Hetero Labs Limited</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>linagliptina</t>
+          <t>enzalutamida</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>25351517487202319</t>
+          <t>25351031614202541</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -1033,7 +1033,7 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>11/08/2026</t>
+          <t>14/08/2026</t>
         </is>
       </c>
     </row>
@@ -1045,12 +1045,12 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>olmesartana medoxomila</t>
+          <t>linagliptina</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>25351454271202416</t>
+          <t>25351517487202319</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -1067,17 +1067,17 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Dr Reddys Farmacêutica Do Brasil Ltda</t>
+          <t>Zhejiang Huahai Pharmaceutical Co., Ltd.</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>naproxeno sódico</t>
+          <t>olmesartana medoxomila</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>25351405623202400</t>
+          <t>25351454271202416</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -1094,17 +1094,17 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Honour Lab Limited</t>
+          <t>Dr Reddys Farmacêutica Do Brasil Ltda</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>cloridrato de fingolimode</t>
+          <t>naproxeno sódico</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>25351650003202253</t>
+          <t>25351405623202400</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -1121,17 +1121,17 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Zydus Lifesciences Limited</t>
+          <t>Honour Lab Limited</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>bromidrato de vortioxetina</t>
+          <t>cloridrato de fingolimode</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>25351141871202590</t>
+          <t>25351650003202253</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -1141,7 +1141,7 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>10/08/2026</t>
+          <t>11/08/2026</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza lista de CADIFAs deferidas (12 novas desde a última execução, 01/09/2026)
</commit_message>
<xml_diff>
--- a/cadifa_completo.xlsx
+++ b/cadifa_completo.xlsx
@@ -7589,7 +7589,7 @@
       </c>
       <c r="D266" t="inlineStr">
         <is>
-          <t>001</t>
+          <t>002</t>
         </is>
       </c>
       <c r="E266" t="inlineStr">
@@ -7886,7 +7886,7 @@
       </c>
       <c r="D277" t="inlineStr">
         <is>
-          <t>001</t>
+          <t>002</t>
         </is>
       </c>
       <c r="E277" t="inlineStr">
@@ -10397,7 +10397,7 @@
       </c>
       <c r="D370" t="inlineStr">
         <is>
-          <t>001</t>
+          <t>002</t>
         </is>
       </c>
       <c r="E370" t="inlineStr">
@@ -12152,7 +12152,7 @@
       </c>
       <c r="D435" t="inlineStr">
         <is>
-          <t>001</t>
+          <t>002</t>
         </is>
       </c>
       <c r="E435" t="inlineStr">
@@ -13070,7 +13070,7 @@
       </c>
       <c r="D469" t="inlineStr">
         <is>
-          <t>001</t>
+          <t>002</t>
         </is>
       </c>
       <c r="E469" t="inlineStr">
@@ -13718,7 +13718,7 @@
       </c>
       <c r="D493" t="inlineStr">
         <is>
-          <t>001</t>
+          <t>002</t>
         </is>
       </c>
       <c r="E493" t="inlineStr">
@@ -14096,7 +14096,7 @@
       </c>
       <c r="D507" t="inlineStr">
         <is>
-          <t>002</t>
+          <t>003</t>
         </is>
       </c>
       <c r="E507" t="inlineStr">
@@ -15581,7 +15581,7 @@
       </c>
       <c r="D562" t="inlineStr">
         <is>
-          <t>001</t>
+          <t>002</t>
         </is>
       </c>
       <c r="E562" t="inlineStr">
@@ -16553,7 +16553,7 @@
       </c>
       <c r="D598" t="inlineStr">
         <is>
-          <t>001</t>
+          <t>002</t>
         </is>
       </c>
       <c r="E598" t="inlineStr">
@@ -16580,7 +16580,7 @@
       </c>
       <c r="D599" t="inlineStr">
         <is>
-          <t>001</t>
+          <t>002</t>
         </is>
       </c>
       <c r="E599" t="inlineStr">
@@ -16715,7 +16715,7 @@
       </c>
       <c r="D604" t="inlineStr">
         <is>
-          <t>001</t>
+          <t>002</t>
         </is>
       </c>
       <c r="E604" t="inlineStr">
@@ -16931,7 +16931,7 @@
       </c>
       <c r="D612" t="inlineStr">
         <is>
-          <t>001</t>
+          <t>002</t>
         </is>
       </c>
       <c r="E612" t="inlineStr">

</xml_diff>

<commit_message>
Atualiza lista de CADIFAs deferidas (2 revisões novas em 08/09/2026)
Novas combinações Nº CADIFA + Revisão desde a última execução:
- 25351145158202272 rev 001.1 (Cipla Limited - dicloridrato de trimetazidina), antes rev 001
- 25351591789202260 rev 002.1 (Biocon Limited - rosuvastatina cálcica), antes rev 002

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AwS4NFerZc63b6Jo3MxYBc
</commit_message>
<xml_diff>
--- a/cadifa_completo.xlsx
+++ b/cadifa_completo.xlsx
@@ -2216,7 +2216,7 @@
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>001</t>
+          <t>001.1</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
@@ -12854,7 +12854,7 @@
       </c>
       <c r="D461" t="inlineStr">
         <is>
-          <t>002</t>
+          <t>002.1</t>
         </is>
       </c>
       <c r="E461" t="inlineStr">

</xml_diff>